<commit_message>
Aggiunto i dtypes delle colonne del csv grezzo e aggiunta l'area di interesse di ogni colonna
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{FD02D6F6-5ABB-44D1-A436-4ED56DDBDB39}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54101D4F-E8B2-204E-94B4-A562D4EC147C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -31,9 +31,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -47,7 +44,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="350">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="361">
   <si>
     <t>gameid</t>
   </si>
@@ -598,9 +595,6 @@
     <t>Posizione e lato della mappa del giocatore</t>
   </si>
   <si>
-    <t>Esempio participantid = 1 indica il toplaner del blue side</t>
-  </si>
-  <si>
     <t>Lato della mappa</t>
   </si>
   <si>
@@ -619,9 +613,6 @@
     <t>ID univoco del team</t>
   </si>
   <si>
-    <t>Indica de il team ha avuto il primo pick</t>
-  </si>
-  <si>
     <t>Campione giocato</t>
   </si>
   <si>
@@ -1097,13 +1088,52 @@
   </si>
   <si>
     <t>Gold Power Rating</t>
+  </si>
+  <si>
+    <t>Esempio: participantid = 1 indica il toplaner del blue side</t>
+  </si>
+  <si>
+    <t>object</t>
+  </si>
+  <si>
+    <t>int64</t>
+  </si>
+  <si>
+    <t>float64</t>
+  </si>
+  <si>
+    <t>Area di interesse</t>
+  </si>
+  <si>
+    <t>Informazioni generali sulla partita</t>
+  </si>
+  <si>
+    <t>Informazioni generali sul giocatore</t>
+  </si>
+  <si>
+    <t>Informazioni generali sul team</t>
+  </si>
+  <si>
+    <t>Indica se il team ha avuto il primo pick</t>
+  </si>
+  <si>
+    <t>Informazioni sulla draft</t>
+  </si>
+  <si>
+    <t>Performance individuale</t>
+  </si>
+  <si>
+    <t>Informazioni generale sul giocatore</t>
+  </si>
+  <si>
+    <t>Performance del team</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="3" x14ac:knownFonts="1">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1123,6 +1153,13 @@
       <sz val="8"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1152,10 +1189,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1490,18 +1528,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
-  <dimension ref="A1:E166"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <dimension ref="A1:F166"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="20.6640625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="6" max="16384" width="8.88671875" style="1"/>
+    <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1517,1394 +1556,2387 @@
       <c r="E1" s="2" t="s">
         <v>177</v>
       </c>
-    </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F1" s="3" t="s">
+        <v>352</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B2" s="1" t="s">
         <v>169</v>
       </c>
-    </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C2" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F2" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B3" s="1" t="s">
         <v>170</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C3" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F3" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B4" s="1" t="s">
         <v>171</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C4" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F4" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B5" s="1" t="s">
         <v>172</v>
       </c>
+      <c r="C5" s="1" t="s">
+        <v>349</v>
+      </c>
       <c r="E5" s="1" t="s">
         <v>180</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F5" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>173</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C6" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F6" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
       <c r="B7" s="1" t="s">
         <v>174</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C7" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F7" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
       <c r="B8" s="1" t="s">
         <v>175</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C8" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
       <c r="B9" s="1" t="s">
         <v>176</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C9" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F9" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>178</v>
       </c>
+      <c r="C10" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E10" s="1" t="s">
         <v>179</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F10" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>181</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F11" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
       <c r="B12" s="1" t="s">
         <v>182</v>
       </c>
+      <c r="C12" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E12" s="1" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.3">
+        <v>348</v>
+      </c>
+      <c r="F12" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.3">
+        <v>183</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F13" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.3">
+        <v>184</v>
+      </c>
+      <c r="C14" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F14" s="1" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+        <v>185</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F15" s="1" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="17" spans="1:2" x14ac:dyDescent="0.3">
+        <v>186</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F16" s="1" t="s">
+        <v>354</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="18" spans="1:2" x14ac:dyDescent="0.3">
+        <v>187</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F17" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="19" spans="1:2" x14ac:dyDescent="0.3">
+        <v>188</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F18" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="20" spans="1:2" x14ac:dyDescent="0.3">
+        <v>356</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F19" s="1" t="s">
+        <v>355</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="21" spans="1:2" x14ac:dyDescent="0.3">
+        <v>189</v>
+      </c>
+      <c r="C20" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F20" s="1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="22" spans="1:2" x14ac:dyDescent="0.3">
+        <v>190</v>
+      </c>
+      <c r="C21" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F21" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="23" spans="1:2" x14ac:dyDescent="0.3">
+        <v>191</v>
+      </c>
+      <c r="C22" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F22" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="24" spans="1:2" x14ac:dyDescent="0.3">
+        <v>192</v>
+      </c>
+      <c r="C23" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F23" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="25" spans="1:2" x14ac:dyDescent="0.3">
+        <v>193</v>
+      </c>
+      <c r="C24" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F24" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="26" spans="1:2" x14ac:dyDescent="0.3">
+        <v>194</v>
+      </c>
+      <c r="C25" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F25" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="27" spans="1:2" x14ac:dyDescent="0.3">
+        <v>195</v>
+      </c>
+      <c r="C26" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F26" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="28" spans="1:2" x14ac:dyDescent="0.3">
+        <v>196</v>
+      </c>
+      <c r="C27" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F27" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="29" spans="1:2" x14ac:dyDescent="0.3">
+        <v>197</v>
+      </c>
+      <c r="C28" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F28" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>200</v>
-      </c>
-    </row>
-    <row r="30" spans="1:2" x14ac:dyDescent="0.3">
+        <v>198</v>
+      </c>
+      <c r="C29" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F29" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>201</v>
-      </c>
-    </row>
-    <row r="31" spans="1:2" x14ac:dyDescent="0.3">
+        <v>199</v>
+      </c>
+      <c r="C30" s="1" t="s">
+        <v>349</v>
+      </c>
+      <c r="F30" s="1" t="s">
+        <v>357</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>202</v>
-      </c>
-    </row>
-    <row r="32" spans="1:2" x14ac:dyDescent="0.3">
+        <v>200</v>
+      </c>
+      <c r="C31" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F31" s="1" t="s">
+        <v>353</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>203</v>
-      </c>
-    </row>
-    <row r="33" spans="1:5" x14ac:dyDescent="0.3">
+        <v>201</v>
+      </c>
+      <c r="C32" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F32" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>204</v>
-      </c>
-    </row>
-    <row r="34" spans="1:5" x14ac:dyDescent="0.3">
+        <v>202</v>
+      </c>
+      <c r="C33" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F33" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>205</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+        <v>203</v>
+      </c>
+      <c r="C34" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F34" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>206</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+        <v>204</v>
+      </c>
+      <c r="C35" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F35" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>207</v>
-      </c>
-    </row>
-    <row r="37" spans="1:5" x14ac:dyDescent="0.3">
+        <v>205</v>
+      </c>
+      <c r="C36" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F36" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>208</v>
-      </c>
-    </row>
-    <row r="38" spans="1:5" x14ac:dyDescent="0.3">
+        <v>206</v>
+      </c>
+      <c r="C37" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F37" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
+      </c>
+      <c r="C38" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E38" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F38" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
+      </c>
+      <c r="C39" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E39" s="1" t="s">
-        <v>214</v>
-      </c>
-    </row>
-    <row r="40" spans="1:5" x14ac:dyDescent="0.3">
+        <v>212</v>
+      </c>
+      <c r="F39" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
+      </c>
+      <c r="C40" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E40" s="1" t="s">
-        <v>215</v>
-      </c>
-    </row>
-    <row r="41" spans="1:5" x14ac:dyDescent="0.3">
+        <v>213</v>
+      </c>
+      <c r="F40" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
+      </c>
+      <c r="C41" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E41" s="1" t="s">
-        <v>216</v>
-      </c>
-    </row>
-    <row r="42" spans="1:5" x14ac:dyDescent="0.3">
+        <v>214</v>
+      </c>
+      <c r="F41" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
+      </c>
+      <c r="C42" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E42" s="1" t="s">
-        <v>221</v>
-      </c>
-    </row>
-    <row r="43" spans="1:5" x14ac:dyDescent="0.3">
+        <v>219</v>
+      </c>
+      <c r="F42" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
+      </c>
+      <c r="C43" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E43" s="1" t="s">
-        <v>222</v>
-      </c>
-    </row>
-    <row r="44" spans="1:5" x14ac:dyDescent="0.3">
+        <v>220</v>
+      </c>
+      <c r="F43" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
+      </c>
+      <c r="C44" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E44" s="1" t="s">
-        <v>223</v>
-      </c>
-    </row>
-    <row r="45" spans="1:5" x14ac:dyDescent="0.3">
+        <v>221</v>
+      </c>
+      <c r="F44" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
+      </c>
+      <c r="C45" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E45" s="1" t="s">
-        <v>224</v>
-      </c>
-    </row>
-    <row r="46" spans="1:5" x14ac:dyDescent="0.3">
+        <v>222</v>
+      </c>
+      <c r="F45" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>225</v>
-      </c>
-    </row>
-    <row r="47" spans="1:5" x14ac:dyDescent="0.3">
+        <v>223</v>
+      </c>
+      <c r="C46" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F46" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
+      </c>
+      <c r="C47" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>227</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+        <v>225</v>
+      </c>
+      <c r="F47" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
+      </c>
+      <c r="C48" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E48" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F48" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>229</v>
-      </c>
-    </row>
-    <row r="50" spans="1:5" x14ac:dyDescent="0.3">
+        <v>227</v>
+      </c>
+      <c r="C49" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F49" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>230</v>
-      </c>
-    </row>
-    <row r="51" spans="1:5" x14ac:dyDescent="0.3">
+        <v>228</v>
+      </c>
+      <c r="C50" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F50" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>231</v>
-      </c>
-    </row>
-    <row r="52" spans="1:5" x14ac:dyDescent="0.3">
+        <v>229</v>
+      </c>
+      <c r="C51" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F51" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>232</v>
-      </c>
-    </row>
-    <row r="53" spans="1:5" x14ac:dyDescent="0.3">
+        <v>230</v>
+      </c>
+      <c r="C52" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F52" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>233</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+        <v>231</v>
+      </c>
+      <c r="C53" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F53" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>234</v>
-      </c>
-    </row>
-    <row r="55" spans="1:5" x14ac:dyDescent="0.3">
+        <v>232</v>
+      </c>
+      <c r="C54" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F54" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>235</v>
-      </c>
-    </row>
-    <row r="56" spans="1:5" x14ac:dyDescent="0.3">
+        <v>233</v>
+      </c>
+      <c r="C55" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F55" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>236</v>
-      </c>
-    </row>
-    <row r="57" spans="1:5" x14ac:dyDescent="0.3">
+        <v>234</v>
+      </c>
+      <c r="C56" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F56" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>237</v>
-      </c>
-    </row>
-    <row r="58" spans="1:5" x14ac:dyDescent="0.3">
+        <v>235</v>
+      </c>
+      <c r="C57" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F57" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>238</v>
-      </c>
-    </row>
-    <row r="59" spans="1:5" x14ac:dyDescent="0.3">
+        <v>236</v>
+      </c>
+      <c r="C58" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F58" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>239</v>
+        <v>237</v>
+      </c>
+      <c r="C59" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>240</v>
-      </c>
-    </row>
-    <row r="60" spans="1:5" x14ac:dyDescent="0.3">
+        <v>238</v>
+      </c>
+      <c r="F59" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>241</v>
-      </c>
-    </row>
-    <row r="61" spans="1:5" x14ac:dyDescent="0.3">
+        <v>239</v>
+      </c>
+      <c r="C60" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F60" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>242</v>
-      </c>
-    </row>
-    <row r="62" spans="1:5" x14ac:dyDescent="0.3">
+        <v>240</v>
+      </c>
+      <c r="C61" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F61" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>243</v>
+        <v>241</v>
+      </c>
+      <c r="C62" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E62" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="63" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F62" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>244</v>
-      </c>
-    </row>
-    <row r="64" spans="1:5" x14ac:dyDescent="0.3">
+        <v>242</v>
+      </c>
+      <c r="C63" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F63" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>245</v>
-      </c>
-    </row>
-    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+        <v>243</v>
+      </c>
+      <c r="C64" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F64" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>246</v>
-      </c>
-    </row>
-    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+        <v>244</v>
+      </c>
+      <c r="C65" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F65" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>247</v>
-      </c>
-    </row>
-    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+        <v>245</v>
+      </c>
+      <c r="C66" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F66" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>248</v>
+        <v>246</v>
+      </c>
+      <c r="C67" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E67" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F67" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>249</v>
-      </c>
-    </row>
-    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+        <v>247</v>
+      </c>
+      <c r="C68" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F68" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>250</v>
-      </c>
-    </row>
-    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+        <v>248</v>
+      </c>
+      <c r="C69" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F69" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>251</v>
+        <v>249</v>
+      </c>
+      <c r="C70" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E70" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F70" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>252</v>
+        <v>250</v>
+      </c>
+      <c r="C71" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E71" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F71" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
+      </c>
+      <c r="C72" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E72" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F72" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>254</v>
-      </c>
-    </row>
-    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+        <v>252</v>
+      </c>
+      <c r="C73" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F73" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>255</v>
-      </c>
-    </row>
-    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+        <v>253</v>
+      </c>
+      <c r="C74" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F74" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
+      </c>
+      <c r="C75" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E75" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F75" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
+      </c>
+      <c r="C76" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E76" s="1" t="s">
-        <v>210</v>
-      </c>
-    </row>
-    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+        <v>208</v>
+      </c>
+      <c r="F76" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>258</v>
-      </c>
-    </row>
-    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+        <v>256</v>
+      </c>
+      <c r="C77" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F77" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>259</v>
-      </c>
-    </row>
-    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+        <v>257</v>
+      </c>
+      <c r="C78" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F78" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>260</v>
-      </c>
-    </row>
-    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+        <v>258</v>
+      </c>
+      <c r="C79" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F79" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>261</v>
-      </c>
-    </row>
-    <row r="81" spans="1:2" x14ac:dyDescent="0.3">
+        <v>259</v>
+      </c>
+      <c r="C80" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F80" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>262</v>
-      </c>
-    </row>
-    <row r="82" spans="1:2" x14ac:dyDescent="0.3">
+        <v>260</v>
+      </c>
+      <c r="C81" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F81" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>263</v>
-      </c>
-    </row>
-    <row r="83" spans="1:2" x14ac:dyDescent="0.3">
+        <v>261</v>
+      </c>
+      <c r="C82" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F82" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>264</v>
-      </c>
-    </row>
-    <row r="84" spans="1:2" x14ac:dyDescent="0.3">
+        <v>262</v>
+      </c>
+      <c r="C83" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F83" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>265</v>
-      </c>
-    </row>
-    <row r="85" spans="1:2" x14ac:dyDescent="0.3">
+        <v>263</v>
+      </c>
+      <c r="C84" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F84" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>266</v>
-      </c>
-    </row>
-    <row r="86" spans="1:2" x14ac:dyDescent="0.3">
+        <v>264</v>
+      </c>
+      <c r="C85" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F85" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>267</v>
-      </c>
-    </row>
-    <row r="87" spans="1:2" x14ac:dyDescent="0.3">
+        <v>265</v>
+      </c>
+      <c r="C86" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F86" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>268</v>
-      </c>
-    </row>
-    <row r="88" spans="1:2" x14ac:dyDescent="0.3">
+        <v>266</v>
+      </c>
+      <c r="C87" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F87" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="89" spans="1:2" x14ac:dyDescent="0.3">
+        <v>267</v>
+      </c>
+      <c r="C88" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F88" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>270</v>
-      </c>
-    </row>
-    <row r="90" spans="1:2" x14ac:dyDescent="0.3">
+        <v>268</v>
+      </c>
+      <c r="C89" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F89" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="91" spans="1:2" x14ac:dyDescent="0.3">
+        <v>269</v>
+      </c>
+      <c r="C90" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F90" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>272</v>
-      </c>
-    </row>
-    <row r="92" spans="1:2" x14ac:dyDescent="0.3">
+        <v>270</v>
+      </c>
+      <c r="C91" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F91" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>273</v>
-      </c>
-    </row>
-    <row r="93" spans="1:2" x14ac:dyDescent="0.3">
+        <v>271</v>
+      </c>
+      <c r="C92" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F92" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>274</v>
-      </c>
-    </row>
-    <row r="94" spans="1:2" x14ac:dyDescent="0.3">
+        <v>272</v>
+      </c>
+      <c r="C93" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F93" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>275</v>
-      </c>
-    </row>
-    <row r="95" spans="1:2" x14ac:dyDescent="0.3">
+        <v>273</v>
+      </c>
+      <c r="C94" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F94" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>276</v>
-      </c>
-    </row>
-    <row r="96" spans="1:2" x14ac:dyDescent="0.3">
+        <v>274</v>
+      </c>
+      <c r="C95" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F95" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>277</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
+        <v>275</v>
+      </c>
+      <c r="C96" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F96" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>278</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
+        <v>276</v>
+      </c>
+      <c r="C97" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F97" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
+        <v>277</v>
+      </c>
+      <c r="C98" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F98" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
+      </c>
+      <c r="C99" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>348</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
+        <v>346</v>
+      </c>
+      <c r="F99" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>280</v>
+        <v>278</v>
+      </c>
+      <c r="C100" s="1" t="s">
+        <v>351</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>349</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
+        <v>347</v>
+      </c>
+      <c r="F100" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>282</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
+        <v>280</v>
+      </c>
+      <c r="C101" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F101" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>283</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+        <v>281</v>
+      </c>
+      <c r="C102" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F102" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>284</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
+        <v>282</v>
+      </c>
+      <c r="C103" s="1" t="s">
+        <v>350</v>
+      </c>
+      <c r="F103" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>285</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
+        <v>283</v>
+      </c>
+      <c r="C104" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F104" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>286</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
+        <v>284</v>
+      </c>
+      <c r="C105" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F105" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>287</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
+        <v>285</v>
+      </c>
+      <c r="C106" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F106" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>288</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
+        <v>286</v>
+      </c>
+      <c r="C107" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F107" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>289</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
+        <v>287</v>
+      </c>
+      <c r="C108" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F108" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
+        <v>288</v>
+      </c>
+      <c r="C109" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F109" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>291</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
+        <v>289</v>
+      </c>
+      <c r="C110" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F110" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>292</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
+        <v>290</v>
+      </c>
+      <c r="C111" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F111" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>293</v>
-      </c>
-    </row>
-    <row r="113" spans="1:2" x14ac:dyDescent="0.3">
+        <v>291</v>
+      </c>
+      <c r="C112" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F112" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>294</v>
-      </c>
-    </row>
-    <row r="114" spans="1:2" x14ac:dyDescent="0.3">
+        <v>292</v>
+      </c>
+      <c r="C113" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F113" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>295</v>
-      </c>
-    </row>
-    <row r="115" spans="1:2" x14ac:dyDescent="0.3">
+        <v>293</v>
+      </c>
+      <c r="C114" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F114" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>296</v>
-      </c>
-    </row>
-    <row r="116" spans="1:2" x14ac:dyDescent="0.3">
+        <v>294</v>
+      </c>
+      <c r="C115" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F115" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>297</v>
-      </c>
-    </row>
-    <row r="117" spans="1:2" x14ac:dyDescent="0.3">
+        <v>295</v>
+      </c>
+      <c r="C116" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F116" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>298</v>
-      </c>
-    </row>
-    <row r="118" spans="1:2" x14ac:dyDescent="0.3">
+        <v>296</v>
+      </c>
+      <c r="C117" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F117" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>299</v>
-      </c>
-    </row>
-    <row r="119" spans="1:2" x14ac:dyDescent="0.3">
+        <v>297</v>
+      </c>
+      <c r="C118" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F118" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>300</v>
-      </c>
-    </row>
-    <row r="120" spans="1:2" x14ac:dyDescent="0.3">
+        <v>298</v>
+      </c>
+      <c r="C119" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F119" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>301</v>
-      </c>
-    </row>
-    <row r="121" spans="1:2" x14ac:dyDescent="0.3">
+        <v>299</v>
+      </c>
+      <c r="C120" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F120" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>302</v>
-      </c>
-    </row>
-    <row r="122" spans="1:2" x14ac:dyDescent="0.3">
+        <v>300</v>
+      </c>
+      <c r="C121" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F121" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>303</v>
-      </c>
-    </row>
-    <row r="123" spans="1:2" x14ac:dyDescent="0.3">
+        <v>301</v>
+      </c>
+      <c r="C122" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F122" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>304</v>
-      </c>
-    </row>
-    <row r="124" spans="1:2" x14ac:dyDescent="0.3">
+        <v>302</v>
+      </c>
+      <c r="C123" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F123" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>305</v>
-      </c>
-    </row>
-    <row r="125" spans="1:2" x14ac:dyDescent="0.3">
+        <v>303</v>
+      </c>
+      <c r="C124" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F124" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="126" spans="1:2" x14ac:dyDescent="0.3">
+        <v>304</v>
+      </c>
+      <c r="C125" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F125" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>307</v>
-      </c>
-    </row>
-    <row r="127" spans="1:2" x14ac:dyDescent="0.3">
+        <v>305</v>
+      </c>
+      <c r="C126" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F126" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>308</v>
-      </c>
-    </row>
-    <row r="128" spans="1:2" x14ac:dyDescent="0.3">
+        <v>306</v>
+      </c>
+      <c r="C127" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F127" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>309</v>
-      </c>
-    </row>
-    <row r="129" spans="1:2" x14ac:dyDescent="0.3">
+        <v>307</v>
+      </c>
+      <c r="C128" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F128" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>310</v>
-      </c>
-    </row>
-    <row r="130" spans="1:2" x14ac:dyDescent="0.3">
+        <v>308</v>
+      </c>
+      <c r="C129" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F129" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="131" spans="1:2" x14ac:dyDescent="0.3">
+        <v>309</v>
+      </c>
+      <c r="C130" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F130" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>312</v>
-      </c>
-    </row>
-    <row r="132" spans="1:2" x14ac:dyDescent="0.3">
+        <v>310</v>
+      </c>
+      <c r="C131" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F131" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>313</v>
-      </c>
-    </row>
-    <row r="133" spans="1:2" x14ac:dyDescent="0.3">
+        <v>311</v>
+      </c>
+      <c r="C132" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F132" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>314</v>
-      </c>
-    </row>
-    <row r="134" spans="1:2" x14ac:dyDescent="0.3">
+        <v>312</v>
+      </c>
+      <c r="C133" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F133" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>315</v>
-      </c>
-    </row>
-    <row r="135" spans="1:2" x14ac:dyDescent="0.3">
+        <v>313</v>
+      </c>
+      <c r="C134" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F134" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>316</v>
-      </c>
-    </row>
-    <row r="136" spans="1:2" x14ac:dyDescent="0.3">
+        <v>314</v>
+      </c>
+      <c r="C135" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F135" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>317</v>
-      </c>
-    </row>
-    <row r="137" spans="1:2" x14ac:dyDescent="0.3">
+        <v>315</v>
+      </c>
+      <c r="C136" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F136" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>318</v>
-      </c>
-    </row>
-    <row r="138" spans="1:2" x14ac:dyDescent="0.3">
+        <v>316</v>
+      </c>
+      <c r="C137" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F137" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>319</v>
-      </c>
-    </row>
-    <row r="139" spans="1:2" x14ac:dyDescent="0.3">
+        <v>317</v>
+      </c>
+      <c r="C138" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F138" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>320</v>
-      </c>
-    </row>
-    <row r="140" spans="1:2" x14ac:dyDescent="0.3">
+        <v>318</v>
+      </c>
+      <c r="C139" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F139" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>321</v>
-      </c>
-    </row>
-    <row r="141" spans="1:2" x14ac:dyDescent="0.3">
+        <v>319</v>
+      </c>
+      <c r="C140" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F140" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>322</v>
-      </c>
-    </row>
-    <row r="142" spans="1:2" x14ac:dyDescent="0.3">
+        <v>320</v>
+      </c>
+      <c r="C141" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F141" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>323</v>
-      </c>
-    </row>
-    <row r="143" spans="1:2" x14ac:dyDescent="0.3">
+        <v>321</v>
+      </c>
+      <c r="C142" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F142" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>324</v>
-      </c>
-    </row>
-    <row r="144" spans="1:2" x14ac:dyDescent="0.3">
+        <v>322</v>
+      </c>
+      <c r="C143" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F143" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>325</v>
-      </c>
-    </row>
-    <row r="145" spans="1:2" x14ac:dyDescent="0.3">
+        <v>323</v>
+      </c>
+      <c r="C144" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F144" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>326</v>
-      </c>
-    </row>
-    <row r="146" spans="1:2" x14ac:dyDescent="0.3">
+        <v>324</v>
+      </c>
+      <c r="C145" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F145" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>327</v>
-      </c>
-    </row>
-    <row r="147" spans="1:2" x14ac:dyDescent="0.3">
+        <v>325</v>
+      </c>
+      <c r="C146" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F146" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>328</v>
-      </c>
-    </row>
-    <row r="148" spans="1:2" x14ac:dyDescent="0.3">
+        <v>326</v>
+      </c>
+      <c r="C147" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F147" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>329</v>
-      </c>
-    </row>
-    <row r="149" spans="1:2" x14ac:dyDescent="0.3">
+        <v>327</v>
+      </c>
+      <c r="C148" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F148" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>330</v>
-      </c>
-    </row>
-    <row r="150" spans="1:2" x14ac:dyDescent="0.3">
+        <v>328</v>
+      </c>
+      <c r="C149" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F149" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>331</v>
-      </c>
-    </row>
-    <row r="151" spans="1:2" x14ac:dyDescent="0.3">
+        <v>329</v>
+      </c>
+      <c r="C150" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F150" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>332</v>
-      </c>
-    </row>
-    <row r="152" spans="1:2" x14ac:dyDescent="0.3">
+        <v>330</v>
+      </c>
+      <c r="C151" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F151" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>333</v>
-      </c>
-    </row>
-    <row r="153" spans="1:2" x14ac:dyDescent="0.3">
+        <v>331</v>
+      </c>
+      <c r="C152" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F152" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>334</v>
-      </c>
-    </row>
-    <row r="154" spans="1:2" x14ac:dyDescent="0.3">
+        <v>332</v>
+      </c>
+      <c r="C153" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F153" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>335</v>
-      </c>
-    </row>
-    <row r="155" spans="1:2" x14ac:dyDescent="0.3">
+        <v>333</v>
+      </c>
+      <c r="C154" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F154" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>336</v>
-      </c>
-    </row>
-    <row r="156" spans="1:2" x14ac:dyDescent="0.3">
+        <v>334</v>
+      </c>
+      <c r="C155" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F155" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>337</v>
-      </c>
-    </row>
-    <row r="157" spans="1:2" x14ac:dyDescent="0.3">
+        <v>335</v>
+      </c>
+      <c r="C156" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F156" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>338</v>
-      </c>
-    </row>
-    <row r="158" spans="1:2" x14ac:dyDescent="0.3">
+        <v>336</v>
+      </c>
+      <c r="C157" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F157" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>339</v>
-      </c>
-    </row>
-    <row r="159" spans="1:2" x14ac:dyDescent="0.3">
+        <v>337</v>
+      </c>
+      <c r="C158" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F158" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>340</v>
-      </c>
-    </row>
-    <row r="160" spans="1:2" x14ac:dyDescent="0.3">
+        <v>338</v>
+      </c>
+      <c r="C159" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F159" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>341</v>
-      </c>
-    </row>
-    <row r="161" spans="1:2" x14ac:dyDescent="0.3">
+        <v>339</v>
+      </c>
+      <c r="C160" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F160" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>342</v>
-      </c>
-    </row>
-    <row r="162" spans="1:2" x14ac:dyDescent="0.3">
+        <v>340</v>
+      </c>
+      <c r="C161" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F161" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>343</v>
-      </c>
-    </row>
-    <row r="163" spans="1:2" x14ac:dyDescent="0.3">
+        <v>341</v>
+      </c>
+      <c r="C162" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F162" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>344</v>
-      </c>
-    </row>
-    <row r="164" spans="1:2" x14ac:dyDescent="0.3">
+        <v>342</v>
+      </c>
+      <c r="C163" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F163" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>345</v>
-      </c>
-    </row>
-    <row r="165" spans="1:2" x14ac:dyDescent="0.3">
+        <v>343</v>
+      </c>
+      <c r="C164" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F164" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>346</v>
-      </c>
-    </row>
-    <row r="166" spans="1:2" x14ac:dyDescent="0.3">
+        <v>344</v>
+      </c>
+      <c r="C165" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F165" s="1" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>347</v>
+        <v>345</v>
+      </c>
+      <c r="C166" s="1" t="s">
+        <v>351</v>
+      </c>
+      <c r="F166" s="1" t="s">
+        <v>358</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
inseriti alcuni dtypes corretti
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10118"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{54101D4F-E8B2-204E-94B4-A562D4EC147C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F56BD1A-40B8-4EB6-9C04-FC934DAA46FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -31,6 +31,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -44,7 +47,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="689" uniqueCount="361">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="364">
   <si>
     <t>gameid</t>
   </si>
@@ -1127,6 +1130,15 @@
   </si>
   <si>
     <t>Performance del team</t>
+  </si>
+  <si>
+    <t>string</t>
+  </si>
+  <si>
+    <t>boolean</t>
+  </si>
+  <si>
+    <t>datetime64</t>
   </si>
 </sst>
 </file>
@@ -1529,18 +1541,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="1"/>
+    <col min="7" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1560,7 +1572,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1570,11 +1582,14 @@
       <c r="C2" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D2" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F2" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1584,11 +1599,14 @@
       <c r="C3" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D3" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F3" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1598,11 +1616,14 @@
       <c r="C4" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D4" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F4" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1612,6 +1633,9 @@
       <c r="C5" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D5" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="E5" s="1" t="s">
         <v>180</v>
       </c>
@@ -1619,7 +1643,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1629,11 +1653,14 @@
       <c r="C6" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D6" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F6" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1643,11 +1670,14 @@
       <c r="C7" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D7" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F7" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1657,11 +1687,14 @@
       <c r="C8" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D8" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="F8" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1671,11 +1704,14 @@
       <c r="C9" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D9" s="1" t="s">
+        <v>363</v>
+      </c>
       <c r="F9" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1685,6 +1721,9 @@
       <c r="C10" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D10" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E10" s="1" t="s">
         <v>179</v>
       </c>
@@ -1692,7 +1731,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1706,7 +1745,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1723,7 +1762,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1737,7 +1776,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1751,7 +1790,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1765,7 +1804,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1779,7 +1818,7 @@
         <v>354</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1793,7 +1832,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -1807,7 +1846,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -1821,7 +1860,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -1835,7 +1874,7 @@
         <v>359</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1849,7 +1888,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -1863,7 +1902,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -1877,7 +1916,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -1891,7 +1930,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -1905,7 +1944,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -1919,7 +1958,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -1933,7 +1972,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -1947,7 +1986,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -1961,7 +2000,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -1975,7 +2014,7 @@
         <v>357</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -1989,7 +2028,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2003,7 +2042,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2017,7 +2056,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2031,7 +2070,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2045,7 +2084,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2059,7 +2098,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2073,7 +2112,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
@@ -2090,7 +2129,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -2107,7 +2146,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
@@ -2124,7 +2163,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
@@ -2141,7 +2180,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2158,7 +2197,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
@@ -2175,7 +2214,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -2192,7 +2231,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
@@ -2209,7 +2248,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -2223,7 +2262,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -2240,7 +2279,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -2257,7 +2296,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -2271,7 +2310,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -2285,7 +2324,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
@@ -2299,7 +2338,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
@@ -2313,7 +2352,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
@@ -2327,7 +2366,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
@@ -2341,7 +2380,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -2355,7 +2394,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -2369,7 +2408,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
@@ -2383,7 +2422,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
@@ -2397,7 +2436,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -2414,7 +2453,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -2428,7 +2467,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
@@ -2442,7 +2481,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -2459,7 +2498,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -2473,7 +2512,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
@@ -2487,7 +2526,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
@@ -2501,7 +2540,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
@@ -2515,7 +2554,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
@@ -2532,7 +2571,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
@@ -2546,7 +2585,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
@@ -2560,7 +2599,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
@@ -2577,7 +2616,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
@@ -2594,7 +2633,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
@@ -2611,7 +2650,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
@@ -2625,7 +2664,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
@@ -2639,7 +2678,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
@@ -2656,7 +2695,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
@@ -2673,7 +2712,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -2687,7 +2726,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
@@ -2701,7 +2740,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
@@ -2715,7 +2754,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
@@ -2729,7 +2768,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
@@ -2743,7 +2782,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
@@ -2757,7 +2796,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
@@ -2771,7 +2810,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -2785,7 +2824,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
@@ -2799,7 +2838,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
@@ -2813,7 +2852,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
@@ -2827,7 +2866,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
@@ -2841,7 +2880,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
@@ -2855,7 +2894,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
@@ -2869,7 +2908,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
@@ -2883,7 +2922,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
@@ -2897,7 +2936,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
@@ -2911,7 +2950,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
@@ -2925,7 +2964,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
@@ -2939,7 +2978,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
@@ -2953,7 +2992,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
@@ -2967,7 +3006,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
@@ -2981,7 +3020,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
@@ -2998,7 +3037,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
@@ -3015,7 +3054,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
@@ -3029,7 +3068,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
@@ -3043,7 +3082,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3057,7 +3096,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
@@ -3071,7 +3110,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
@@ -3085,7 +3124,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
@@ -3099,7 +3138,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
@@ -3113,7 +3152,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
@@ -3127,7 +3166,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
@@ -3141,7 +3180,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
@@ -3155,7 +3194,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
@@ -3169,7 +3208,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
@@ -3183,7 +3222,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
@@ -3197,7 +3236,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
@@ -3211,7 +3250,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
@@ -3225,7 +3264,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
@@ -3239,7 +3278,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
@@ -3253,7 +3292,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
@@ -3267,7 +3306,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -3281,7 +3320,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -3295,7 +3334,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
@@ -3309,7 +3348,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
@@ -3323,7 +3362,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
@@ -3337,7 +3376,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
@@ -3351,7 +3390,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
@@ -3365,7 +3404,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
@@ -3379,7 +3418,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
@@ -3393,7 +3432,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
@@ -3407,7 +3446,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
@@ -3421,7 +3460,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
@@ -3435,7 +3474,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
@@ -3449,7 +3488,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
@@ -3463,7 +3502,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
@@ -3477,7 +3516,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
@@ -3491,7 +3530,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
@@ -3505,7 +3544,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
@@ -3519,7 +3558,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
@@ -3533,7 +3572,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
@@ -3547,7 +3586,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
@@ -3561,7 +3600,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
@@ -3575,7 +3614,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
@@ -3589,7 +3628,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
@@ -3603,7 +3642,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
@@ -3617,7 +3656,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
@@ -3631,7 +3670,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
@@ -3645,7 +3684,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -3659,7 +3698,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
@@ -3673,7 +3712,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
@@ -3687,7 +3726,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
@@ -3701,7 +3740,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
@@ -3715,7 +3754,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
@@ -3729,7 +3768,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
@@ -3743,7 +3782,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
@@ -3757,7 +3796,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
@@ -3771,7 +3810,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
@@ -3785,7 +3824,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -3799,7 +3838,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
@@ -3813,7 +3852,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
@@ -3827,7 +3866,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
@@ -3841,7 +3880,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
@@ -3855,7 +3894,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
@@ -3869,7 +3908,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
@@ -3883,7 +3922,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
@@ -3897,7 +3936,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
@@ -3911,7 +3950,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
@@ -3925,7 +3964,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>

</xml_diff>

<commit_message>
scritti i dtypes appropriati sul file metadati e crate schede guida per analisi di team e individuali
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,19 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3F56BD1A-40B8-4EB6-9C04-FC934DAA46FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1402B7A7-A4BB-FC40-9B75-95AC633BA5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" activeTab="2" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
+    <sheet name="Analisi performance di team" sheetId="2" r:id="rId2"/>
+    <sheet name="Analisi performance individuali" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -31,9 +33,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -47,7 +46,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="698" uniqueCount="364">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="365">
   <si>
     <t>gameid</t>
   </si>
@@ -1139,6 +1138,9 @@
   </si>
   <si>
     <t>datetime64</t>
+  </si>
+  <si>
+    <t>???</t>
   </si>
 </sst>
 </file>
@@ -1541,18 +1543,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.77734375" style="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1572,7 +1574,7 @@
         <v>352</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1589,7 +1591,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1606,7 +1608,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1623,7 +1625,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1643,7 +1645,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1660,7 +1662,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1677,7 +1679,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1694,7 +1696,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1711,7 +1713,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1731,7 +1733,7 @@
         <v>353</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1741,11 +1743,14 @@
       <c r="C11" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D11" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F11" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1755,6 +1760,9 @@
       <c r="C12" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D12" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E12" s="1" t="s">
         <v>348</v>
       </c>
@@ -1762,7 +1770,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1772,11 +1780,14 @@
       <c r="C13" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D13" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F13" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1786,11 +1797,14 @@
       <c r="C14" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D14" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F14" s="1" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1800,11 +1814,14 @@
       <c r="C15" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D15" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F15" s="1" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1814,11 +1831,14 @@
       <c r="C16" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D16" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F16" s="1" t="s">
         <v>354</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1828,11 +1848,14 @@
       <c r="C17" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D17" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F17" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -1842,11 +1865,14 @@
       <c r="C18" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D18" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F18" s="1" t="s">
         <v>355</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -1860,7 +1886,7 @@
         <v>355</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -1870,11 +1896,14 @@
       <c r="C20" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D20" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F20" s="1" t="s">
         <v>359</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1884,11 +1913,14 @@
       <c r="C21" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D21" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F21" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -1898,11 +1930,14 @@
       <c r="C22" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D22" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F22" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -1912,11 +1947,14 @@
       <c r="C23" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D23" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F23" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -1926,11 +1964,14 @@
       <c r="C24" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D24" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F24" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -1940,11 +1981,14 @@
       <c r="C25" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D25" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F25" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -1954,11 +1998,14 @@
       <c r="C26" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D26" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F26" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -1968,11 +2015,14 @@
       <c r="C27" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D27" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F27" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -1982,11 +2032,14 @@
       <c r="C28" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D28" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F28" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -1996,11 +2049,14 @@
       <c r="C29" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D29" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F29" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -2010,11 +2066,14 @@
       <c r="C30" s="1" t="s">
         <v>349</v>
       </c>
+      <c r="D30" s="1" t="s">
+        <v>361</v>
+      </c>
       <c r="F30" s="1" t="s">
         <v>357</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2024,11 +2083,14 @@
       <c r="C31" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D31" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F31" s="1" t="s">
         <v>353</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2038,11 +2100,14 @@
       <c r="C32" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D32" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="F32" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2052,11 +2117,14 @@
       <c r="C33" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D33" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F33" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2066,11 +2134,14 @@
       <c r="C34" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D34" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F34" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2080,11 +2151,14 @@
       <c r="C35" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D35" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F35" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2094,11 +2168,14 @@
       <c r="C36" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D36" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F36" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2108,11 +2185,14 @@
       <c r="C37" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D37" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F37" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
@@ -2122,6 +2202,9 @@
       <c r="C38" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D38" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E38" s="1" t="s">
         <v>208</v>
       </c>
@@ -2129,7 +2212,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -2139,6 +2222,9 @@
       <c r="C39" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D39" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E39" s="1" t="s">
         <v>212</v>
       </c>
@@ -2146,7 +2232,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
@@ -2156,6 +2242,9 @@
       <c r="C40" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D40" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E40" s="1" t="s">
         <v>213</v>
       </c>
@@ -2163,7 +2252,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
@@ -2173,6 +2262,9 @@
       <c r="C41" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D41" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="E41" s="1" t="s">
         <v>214</v>
       </c>
@@ -2180,7 +2272,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2190,6 +2282,9 @@
       <c r="C42" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D42" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E42" s="1" t="s">
         <v>219</v>
       </c>
@@ -2197,7 +2292,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
@@ -2207,6 +2302,9 @@
       <c r="C43" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D43" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E43" s="1" t="s">
         <v>220</v>
       </c>
@@ -2214,7 +2312,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -2224,6 +2322,9 @@
       <c r="C44" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D44" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E44" s="1" t="s">
         <v>221</v>
       </c>
@@ -2231,7 +2332,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
@@ -2241,6 +2342,9 @@
       <c r="C45" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D45" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E45" s="1" t="s">
         <v>222</v>
       </c>
@@ -2248,7 +2352,7 @@
         <v>358</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -2258,11 +2362,14 @@
       <c r="C46" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D46" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F46" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -2272,6 +2379,9 @@
       <c r="C47" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D47" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="E47" s="1" t="s">
         <v>225</v>
       </c>
@@ -2279,7 +2389,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -2289,6 +2399,9 @@
       <c r="C48" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D48" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E48" s="1" t="s">
         <v>208</v>
       </c>
@@ -2296,7 +2409,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -2306,11 +2419,14 @@
       <c r="C49" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D49" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F49" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -2320,11 +2436,14 @@
       <c r="C50" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D50" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F50" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
@@ -2334,11 +2453,14 @@
       <c r="C51" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D51" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F51" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
@@ -2348,11 +2470,14 @@
       <c r="C52" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D52" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F52" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
@@ -2362,11 +2487,14 @@
       <c r="C53" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D53" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F53" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
@@ -2376,11 +2504,14 @@
       <c r="C54" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D54" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F54" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -2390,11 +2521,14 @@
       <c r="C55" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D55" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F55" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -2404,11 +2538,14 @@
       <c r="C56" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D56" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F56" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
@@ -2418,11 +2555,14 @@
       <c r="C57" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D57" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F57" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
@@ -2432,11 +2572,14 @@
       <c r="C58" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D58" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F58" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -2446,6 +2589,9 @@
       <c r="C59" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D59" s="1" t="s">
+        <v>364</v>
+      </c>
       <c r="E59" s="1" t="s">
         <v>238</v>
       </c>
@@ -2453,7 +2599,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -2463,11 +2609,14 @@
       <c r="C60" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D60" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F60" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
@@ -2477,11 +2626,14 @@
       <c r="C61" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D61" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F61" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -2491,6 +2643,9 @@
       <c r="C62" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D62" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E62" s="1" t="s">
         <v>208</v>
       </c>
@@ -2498,7 +2653,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -2508,11 +2663,14 @@
       <c r="C63" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D63" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F63" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
@@ -2522,11 +2680,14 @@
       <c r="C64" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D64" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F64" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
@@ -2536,11 +2697,14 @@
       <c r="C65" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D65" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F65" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
@@ -2550,11 +2714,14 @@
       <c r="C66" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D66" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F66" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
@@ -2564,6 +2731,9 @@
       <c r="C67" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D67" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E67" s="1" t="s">
         <v>208</v>
       </c>
@@ -2571,7 +2741,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
@@ -2581,11 +2751,14 @@
       <c r="C68" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D68" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F68" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
@@ -2595,11 +2768,14 @@
       <c r="C69" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D69" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F69" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
@@ -2609,6 +2785,9 @@
       <c r="C70" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D70" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E70" s="1" t="s">
         <v>208</v>
       </c>
@@ -2616,7 +2795,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
@@ -2626,6 +2805,9 @@
       <c r="C71" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D71" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E71" s="1" t="s">
         <v>208</v>
       </c>
@@ -2633,7 +2815,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
@@ -2643,6 +2825,9 @@
       <c r="C72" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D72" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E72" s="1" t="s">
         <v>208</v>
       </c>
@@ -2650,7 +2835,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
@@ -2660,11 +2845,14 @@
       <c r="C73" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D73" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F73" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
@@ -2674,11 +2862,14 @@
       <c r="C74" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D74" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F74" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
@@ -2688,6 +2879,9 @@
       <c r="C75" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D75" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E75" s="1" t="s">
         <v>208</v>
       </c>
@@ -2695,7 +2889,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
@@ -2705,6 +2899,9 @@
       <c r="C76" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D76" s="1" t="s">
+        <v>362</v>
+      </c>
       <c r="E76" s="1" t="s">
         <v>208</v>
       </c>
@@ -2712,7 +2909,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -2722,11 +2919,14 @@
       <c r="C77" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D77" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F77" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
@@ -2736,11 +2936,14 @@
       <c r="C78" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D78" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F78" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
@@ -2750,11 +2953,14 @@
       <c r="C79" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D79" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F79" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
@@ -2764,11 +2970,14 @@
       <c r="C80" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D80" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F80" s="1" t="s">
         <v>360</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
@@ -2778,11 +2987,14 @@
       <c r="C81" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D81" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F81" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
@@ -2792,11 +3004,14 @@
       <c r="C82" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D82" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F82" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
@@ -2806,11 +3021,14 @@
       <c r="C83" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D83" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F83" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -2820,11 +3038,14 @@
       <c r="C84" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D84" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F84" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
@@ -2834,11 +3055,14 @@
       <c r="C85" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D85" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F85" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
@@ -2848,11 +3072,14 @@
       <c r="C86" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D86" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F86" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
@@ -2862,11 +3089,14 @@
       <c r="C87" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D87" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F87" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
@@ -2876,11 +3106,14 @@
       <c r="C88" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D88" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F88" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
@@ -2890,11 +3123,14 @@
       <c r="C89" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D89" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F89" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
@@ -2904,11 +3140,14 @@
       <c r="C90" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D90" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F90" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
@@ -2918,11 +3157,14 @@
       <c r="C91" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D91" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F91" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
@@ -2932,11 +3174,14 @@
       <c r="C92" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D92" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F92" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
@@ -2946,11 +3191,14 @@
       <c r="C93" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D93" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F93" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
@@ -2960,11 +3208,14 @@
       <c r="C94" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D94" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F94" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
@@ -2974,11 +3225,14 @@
       <c r="C95" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D95" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F95" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
@@ -2988,11 +3242,14 @@
       <c r="C96" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D96" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F96" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
@@ -3002,11 +3259,14 @@
       <c r="C97" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D97" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F97" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
@@ -3016,11 +3276,14 @@
       <c r="C98" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D98" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F98" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
@@ -3030,6 +3293,9 @@
       <c r="C99" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D99" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="E99" s="1" t="s">
         <v>346</v>
       </c>
@@ -3037,7 +3303,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
@@ -3047,6 +3313,9 @@
       <c r="C100" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D100" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="E100" s="1" t="s">
         <v>347</v>
       </c>
@@ -3054,7 +3323,7 @@
         <v>360</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
@@ -3064,11 +3333,14 @@
       <c r="C101" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D101" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F101" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
@@ -3078,11 +3350,14 @@
       <c r="C102" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D102" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F102" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3092,11 +3367,14 @@
       <c r="C103" s="1" t="s">
         <v>350</v>
       </c>
+      <c r="D103" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F103" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
@@ -3106,11 +3384,14 @@
       <c r="C104" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D104" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F104" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
@@ -3120,11 +3401,14 @@
       <c r="C105" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D105" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F105" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
@@ -3134,11 +3418,14 @@
       <c r="C106" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D106" s="1" t="s">
+        <v>351</v>
+      </c>
       <c r="F106" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
@@ -3148,11 +3435,14 @@
       <c r="C107" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D107" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F107" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
@@ -3162,11 +3452,14 @@
       <c r="C108" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D108" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F108" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
@@ -3176,11 +3469,14 @@
       <c r="C109" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D109" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F109" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
@@ -3190,11 +3486,14 @@
       <c r="C110" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D110" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F110" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
@@ -3204,11 +3503,14 @@
       <c r="C111" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D111" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F111" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
@@ -3218,11 +3520,14 @@
       <c r="C112" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D112" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F112" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
@@ -3232,11 +3537,14 @@
       <c r="C113" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D113" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F113" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
@@ -3246,11 +3554,14 @@
       <c r="C114" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D114" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F114" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
@@ -3260,11 +3571,14 @@
       <c r="C115" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D115" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F115" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
@@ -3274,11 +3588,14 @@
       <c r="C116" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D116" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F116" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
@@ -3288,11 +3605,14 @@
       <c r="C117" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D117" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F117" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
@@ -3302,11 +3622,14 @@
       <c r="C118" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D118" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F118" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -3316,11 +3639,14 @@
       <c r="C119" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D119" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F119" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -3330,11 +3656,14 @@
       <c r="C120" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D120" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F120" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
@@ -3344,11 +3673,14 @@
       <c r="C121" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D121" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F121" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
@@ -3358,11 +3690,14 @@
       <c r="C122" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D122" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F122" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
@@ -3372,11 +3707,14 @@
       <c r="C123" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D123" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F123" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
@@ -3386,11 +3724,14 @@
       <c r="C124" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D124" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F124" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
@@ -3400,11 +3741,14 @@
       <c r="C125" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D125" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F125" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
@@ -3414,11 +3758,14 @@
       <c r="C126" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D126" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F126" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
@@ -3428,11 +3775,14 @@
       <c r="C127" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D127" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F127" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
@@ -3442,11 +3792,14 @@
       <c r="C128" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D128" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F128" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
@@ -3456,11 +3809,14 @@
       <c r="C129" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D129" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F129" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
@@ -3470,11 +3826,14 @@
       <c r="C130" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D130" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F130" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
@@ -3484,11 +3843,14 @@
       <c r="C131" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D131" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F131" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
@@ -3498,11 +3860,14 @@
       <c r="C132" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D132" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F132" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
@@ -3512,11 +3877,14 @@
       <c r="C133" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D133" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F133" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
@@ -3526,11 +3894,14 @@
       <c r="C134" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D134" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F134" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
@@ -3540,11 +3911,14 @@
       <c r="C135" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D135" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F135" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
@@ -3554,11 +3928,14 @@
       <c r="C136" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D136" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F136" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
@@ -3568,11 +3945,14 @@
       <c r="C137" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D137" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F137" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
@@ -3582,11 +3962,14 @@
       <c r="C138" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D138" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F138" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
@@ -3596,11 +3979,14 @@
       <c r="C139" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D139" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F139" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
@@ -3610,11 +3996,14 @@
       <c r="C140" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D140" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F140" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
@@ -3624,11 +4013,14 @@
       <c r="C141" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D141" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F141" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
@@ -3638,11 +4030,14 @@
       <c r="C142" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D142" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F142" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
@@ -3652,11 +4047,14 @@
       <c r="C143" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D143" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F143" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
@@ -3666,11 +4064,14 @@
       <c r="C144" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D144" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F144" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
@@ -3680,11 +4081,14 @@
       <c r="C145" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D145" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F145" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -3694,11 +4098,14 @@
       <c r="C146" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D146" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F146" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
@@ -3708,11 +4115,14 @@
       <c r="C147" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D147" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F147" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
@@ -3722,11 +4132,14 @@
       <c r="C148" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D148" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F148" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
@@ -3736,11 +4149,14 @@
       <c r="C149" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D149" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F149" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
@@ -3750,11 +4166,14 @@
       <c r="C150" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D150" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F150" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
@@ -3764,11 +4183,14 @@
       <c r="C151" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D151" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F151" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
@@ -3778,11 +4200,14 @@
       <c r="C152" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D152" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F152" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
@@ -3792,11 +4217,14 @@
       <c r="C153" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D153" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F153" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
@@ -3806,11 +4234,14 @@
       <c r="C154" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D154" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F154" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
@@ -3820,11 +4251,14 @@
       <c r="C155" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D155" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F155" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -3834,11 +4268,14 @@
       <c r="C156" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D156" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F156" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
@@ -3848,11 +4285,14 @@
       <c r="C157" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D157" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F157" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
@@ -3862,11 +4302,14 @@
       <c r="C158" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D158" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F158" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
@@ -3876,11 +4319,14 @@
       <c r="C159" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D159" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F159" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
@@ -3890,11 +4336,14 @@
       <c r="C160" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D160" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F160" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
@@ -3904,11 +4353,14 @@
       <c r="C161" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D161" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F161" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
@@ -3918,11 +4370,14 @@
       <c r="C162" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D162" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F162" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
@@ -3932,11 +4387,14 @@
       <c r="C163" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D163" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F163" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
@@ -3946,11 +4404,14 @@
       <c r="C164" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D164" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F164" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
@@ -3960,11 +4421,14 @@
       <c r="C165" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D165" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F165" s="1" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
@@ -3974,12 +4438,39 @@
       <c r="C166" s="1" t="s">
         <v>351</v>
       </c>
+      <c r="D166" s="1" t="s">
+        <v>350</v>
+      </c>
       <c r="F166" s="1" t="s">
         <v>358</v>
       </c>
     </row>
   </sheetData>
   <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
+  <dimension ref="A1"/>
+  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <cols>
+    <col min="1" max="16384" width="10.83203125" style="1"/>
+  </cols>
+  <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
stabilito le domande su cui sviluppare il progetto
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,21 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{1402B7A7-A4BB-FC40-9B75-95AC633BA5EE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7049A00-E799-4FA5-BB81-B16E4B5CE4D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" activeTab="2" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
-    <sheet name="Analisi performance di team" sheetId="2" r:id="rId2"/>
-    <sheet name="Analisi performance individuali" sheetId="3" r:id="rId3"/>
+    <sheet name="Analisi generali" sheetId="5" r:id="rId2"/>
+    <sheet name="Analisi performance di team" sheetId="2" r:id="rId3"/>
+    <sheet name="Analisi performance individuali" sheetId="3" r:id="rId4"/>
+    <sheet name="Domande avanzate" sheetId="6" r:id="rId5"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -33,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -46,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="853" uniqueCount="365">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="404">
   <si>
     <t>gameid</t>
   </si>
@@ -669,30 +674,9 @@
     <t>Morti totali del team</t>
   </si>
   <si>
-    <t>Se il giocatore ha effettuato una uccisione doppia</t>
-  </si>
-  <si>
     <t>1 = SI ; 0 = NO</t>
   </si>
   <si>
-    <t>Se il giocatore ha effettuato una uccisione tripla</t>
-  </si>
-  <si>
-    <t>Se il giocatore ha effettuato una uccisione quadra</t>
-  </si>
-  <si>
-    <t>Se il giocatore ha effettuato una uccisione penta</t>
-  </si>
-  <si>
-    <t>2 = SI ; 0 = NO</t>
-  </si>
-  <si>
-    <t>3 = SI ; 0 = NO</t>
-  </si>
-  <si>
-    <t>4 = SI ; 0 = NO</t>
-  </si>
-  <si>
     <t>Se il giocatore è stato coinvolto nel primo sangue</t>
   </si>
   <si>
@@ -705,18 +689,6 @@
     <t>Se il giocatore è stato la vittima del primo sangue</t>
   </si>
   <si>
-    <t>5 = SI ; 0 = NO</t>
-  </si>
-  <si>
-    <t>6 = SI ; 0 = NO</t>
-  </si>
-  <si>
-    <t>7 = SI ; 0 = NO</t>
-  </si>
-  <si>
-    <t>8 = SI ; 0 = NO</t>
-  </si>
-  <si>
     <t>Uccisioni per minuto del team</t>
   </si>
   <si>
@@ -1141,6 +1113,430 @@
   </si>
   <si>
     <t>???</t>
+  </si>
+  <si>
+    <t>Quante uccisioni penta ha ottenuto il giocatore</t>
+  </si>
+  <si>
+    <t>Quante uccisioni doppie ha ottenuto il giocatore</t>
+  </si>
+  <si>
+    <t>Quante uccisioni triple ha ottenuto il giocatore</t>
+  </si>
+  <si>
+    <t>Quante uccisioni quadra ha ottenuto il giocatore</t>
+  </si>
+  <si>
+    <t>Contesto competitivo</t>
+  </si>
+  <si>
+    <t>Quante partite sono state giocate nel LEC nel 2025 e con quale distribuzione per split (Spring / Summer / Finals)?</t>
+  </si>
+  <si>
+    <t>Qual è la durata media delle partite LEC nel 2025?</t>
+  </si>
+  <si>
+    <t>La durata media delle partite LEC  è variata nei vari split??</t>
+  </si>
+  <si>
+    <r>
+      <t>Qual è la percentuale di vittorie BLUE SIDE</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> </t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vs RED SIDE nel LEC 2025?</t>
+    </r>
+  </si>
+  <si>
+    <t>Esiste una correlazione tra durata della partita e probabilità di vittoria?</t>
+  </si>
+  <si>
+    <t>Meta &amp; ritmo di gioco</t>
+  </si>
+  <si>
+    <t>Qual è il numero medio di kill per partita nel LEC 2025?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Le partite del LEC 2025 sono più </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>early-game oriented</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> o </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>late-game oriented</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <t>Quanto incide mediamente la first blood sull’esito finale?</t>
+  </si>
+  <si>
+    <t>Qual è la frequenza di partite “snowball” (vantaggio gold &gt; X entro 15 minuti)?</t>
+  </si>
+  <si>
+    <t>Obiettivi neutrali</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Ottenere il </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>first Baron</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> aumenta significativamente la probabilità di vittoria?</t>
+    </r>
+  </si>
+  <si>
+    <t>Quante partite vengono chiuse senza Baron o senza Dragon Soul?</t>
+  </si>
+  <si>
+    <t>Efficienza e macro</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quali team del LEC hanno il </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gold difference medio più alto a 15 minuti</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Esiste una relazione tra </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gold diff @15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> e win rate finale del team?</t>
+    </r>
+  </si>
+  <si>
+    <t>Quali team convertono meglio il vantaggio iniziale in vittoria?</t>
+  </si>
+  <si>
+    <t>Quali team recuperano più spesso partite partendo in svantaggio?</t>
+  </si>
+  <si>
+    <t>Obiettivi e controllo mappa</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quali team hanno il miglior </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>dragon control rate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quali team hanno il miglior </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Baron conversion rate</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> (Baron → win)?</t>
+    </r>
+  </si>
+  <si>
+    <t>Quali team prendono più torri nei primi 20 minuti?</t>
+  </si>
+  <si>
+    <t>Il controllo della vision (wards piazzate / distrutte) è associato a una win rate più alta?</t>
+  </si>
+  <si>
+    <t>Stile di gioco</t>
+  </si>
+  <si>
+    <t>Quali team giocano partite mediamente più lunghe?</t>
+  </si>
+  <si>
+    <t>Quali team hanno uno stile più aggressivo (kills/min, deaths/min)?</t>
+  </si>
+  <si>
+    <t>Esistono team “low kill – high objective efficiency”?</t>
+  </si>
+  <si>
+    <t>Performance per ruolo</t>
+  </si>
+  <si>
+    <t>Quali jungler partecipano alla percentuale più alta di kill del team (KP%)?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quali support hanno il miglior </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>vision score per minuto</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quali giocatori hanno il miglior </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>gold diff @15</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> nel LEC 2025?</t>
+    </r>
+  </si>
+  <si>
+    <t>Quale ruolo  ha il miglior damage share medio?</t>
+  </si>
+  <si>
+    <t>Impatto sulla vittoria</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Esiste una correlazione tra </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>KDA individuale</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> e win rate?</t>
+    </r>
+  </si>
+  <si>
+    <t>Quali giocatori hanno il maggiore impatto nei primi 15 minuti?</t>
+  </si>
+  <si>
+    <t>I giocatori con alto damage share vincono più partite?</t>
+  </si>
+  <si>
+    <t>Consistenza</t>
+  </si>
+  <si>
+    <t>Quali giocatori mantengono performance stabili per tutta la stagione?</t>
+  </si>
+  <si>
+    <t>Quali player hanno la maggiore varianza di performance (partite molto buone vs molto negative)?</t>
+  </si>
+  <si>
+    <t>Esistono player “clutch” con migliori performance nelle partite lunghe (&gt;35 min)?</t>
+  </si>
+  <si>
+    <t>Domande avanzate</t>
+  </si>
+  <si>
+    <t>Quali metriche spiegano meglio la vittoria nel LEC 2025? (feature importance)</t>
+  </si>
+  <si>
+    <t>È possibile costruire un modello predittivo della vittoria usando solo dati @15 minuti?</t>
+  </si>
+  <si>
+    <t>Le metriche di team spiegano la vittoria meglio delle metriche individuali?</t>
+  </si>
+  <si>
+    <r>
+      <t xml:space="preserve">Quali giocatori performano meglio </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>indipendentemente dal team</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color theme="1"/>
+        <rFont val="Aptos Narrow"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>?</t>
+    </r>
   </si>
 </sst>
 </file>
@@ -1203,11 +1599,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1543,18 +1940,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.1640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="17.109375" style="1" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="1"/>
+    <col min="7" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1571,10 +1968,10 @@
         <v>177</v>
       </c>
       <c r="F1" s="3" t="s">
-        <v>352</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+        <v>341</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1582,16 +1979,16 @@
         <v>169</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F2" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1599,16 +1996,16 @@
         <v>170</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F3" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1616,16 +2013,16 @@
         <v>171</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F4" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -1633,19 +2030,19 @@
         <v>172</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="E5" s="1" t="s">
         <v>180</v>
       </c>
       <c r="F5" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -1653,16 +2050,16 @@
         <v>173</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F6" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -1670,16 +2067,16 @@
         <v>174</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F7" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -1687,16 +2084,16 @@
         <v>175</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="F8" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -1704,16 +2101,16 @@
         <v>176</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>363</v>
+        <v>352</v>
       </c>
       <c r="F9" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -1721,19 +2118,19 @@
         <v>178</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="E10" s="1" t="s">
         <v>179</v>
       </c>
       <c r="F10" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -1741,16 +2138,16 @@
         <v>181</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F11" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -1758,19 +2155,19 @@
         <v>182</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D12" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="E12" s="1" t="s">
-        <v>348</v>
+        <v>337</v>
       </c>
       <c r="F12" s="1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -1778,16 +2175,16 @@
         <v>183</v>
       </c>
       <c r="C13" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D13" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F13" s="1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -1795,16 +2192,16 @@
         <v>184</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D14" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F14" s="1" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -1812,16 +2209,16 @@
         <v>185</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D15" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F15" s="1" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -1829,16 +2226,16 @@
         <v>186</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D16" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F16" s="1" t="s">
-        <v>354</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+        <v>343</v>
+      </c>
+    </row>
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -1846,16 +2243,16 @@
         <v>187</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D17" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F17" s="1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -1863,30 +2260,33 @@
         <v>188</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D18" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F18" s="1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>356</v>
+        <v>345</v>
       </c>
       <c r="C19" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D19" s="1" t="s">
         <v>351</v>
       </c>
       <c r="F19" s="1" t="s">
-        <v>355</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+        <v>344</v>
+      </c>
+    </row>
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -1894,16 +2294,16 @@
         <v>189</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D20" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F20" s="1" t="s">
-        <v>359</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+        <v>348</v>
+      </c>
+    </row>
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -1911,16 +2311,16 @@
         <v>190</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D21" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F21" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -1928,16 +2328,16 @@
         <v>191</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D22" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F22" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -1945,16 +2345,16 @@
         <v>192</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D23" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F23" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -1962,16 +2362,16 @@
         <v>193</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D24" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F24" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -1979,16 +2379,16 @@
         <v>194</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D25" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F25" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -1996,16 +2396,16 @@
         <v>195</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D26" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F26" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -2013,16 +2413,16 @@
         <v>196</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D27" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F27" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -2030,16 +2430,16 @@
         <v>197</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D28" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F28" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -2047,16 +2447,16 @@
         <v>198</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D29" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F29" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -2064,16 +2464,16 @@
         <v>199</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>349</v>
+        <v>338</v>
       </c>
       <c r="D30" s="1" t="s">
-        <v>361</v>
+        <v>350</v>
       </c>
       <c r="F30" s="1" t="s">
-        <v>357</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+        <v>346</v>
+      </c>
+    </row>
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2081,16 +2481,16 @@
         <v>200</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D31" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F31" s="1" t="s">
-        <v>353</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+        <v>342</v>
+      </c>
+    </row>
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2098,16 +2498,16 @@
         <v>201</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D32" s="1" t="s">
-        <v>362</v>
+        <v>351</v>
       </c>
       <c r="F32" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2115,16 +2515,16 @@
         <v>202</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D33" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F33" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2132,16 +2532,16 @@
         <v>203</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D34" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F34" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2149,16 +2549,16 @@
         <v>204</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D35" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F35" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2166,16 +2566,16 @@
         <v>205</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D36" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F36" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2183,2266 +2583,2254 @@
         <v>206</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D37" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F37" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>207</v>
+        <v>355</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D38" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="E38" s="1" t="s">
-        <v>208</v>
+        <v>339</v>
       </c>
       <c r="F38" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>209</v>
+        <v>356</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D39" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="E39" s="1" t="s">
-        <v>212</v>
+        <v>339</v>
       </c>
       <c r="F39" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>210</v>
+        <v>357</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D40" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="E40" s="1" t="s">
-        <v>213</v>
+        <v>339</v>
       </c>
       <c r="F40" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>211</v>
+        <v>354</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D41" s="1" t="s">
-        <v>350</v>
-      </c>
-      <c r="E41" s="1" t="s">
-        <v>214</v>
+        <v>339</v>
       </c>
       <c r="F41" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>215</v>
+        <v>208</v>
       </c>
       <c r="C42" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D42" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D42" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E42" s="1" t="s">
-        <v>219</v>
+        <v>207</v>
       </c>
       <c r="F42" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>217</v>
+        <v>210</v>
       </c>
       <c r="C43" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D43" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D43" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E43" s="1" t="s">
-        <v>220</v>
+        <v>207</v>
       </c>
       <c r="F43" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>216</v>
+        <v>209</v>
       </c>
       <c r="C44" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D44" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D44" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E44" s="1" t="s">
-        <v>221</v>
+        <v>207</v>
       </c>
       <c r="F44" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>218</v>
+        <v>211</v>
       </c>
       <c r="C45" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D45" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D45" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E45" s="1" t="s">
-        <v>222</v>
+        <v>207</v>
       </c>
       <c r="F45" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>223</v>
+        <v>212</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D46" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F46" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>224</v>
+        <v>213</v>
       </c>
       <c r="C47" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D47" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="E47" s="1" t="s">
-        <v>225</v>
+        <v>214</v>
       </c>
       <c r="F47" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>226</v>
+        <v>215</v>
       </c>
       <c r="C48" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D48" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D48" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E48" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F48" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>227</v>
+        <v>216</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D49" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F49" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>228</v>
+        <v>217</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D50" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F50" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>229</v>
+        <v>218</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D51" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F51" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>230</v>
+        <v>219</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D52" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F52" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>231</v>
+        <v>220</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D53" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F53" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>232</v>
+        <v>221</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D54" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F54" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>233</v>
+        <v>222</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D55" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F55" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>234</v>
+        <v>223</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D56" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F56" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>235</v>
+        <v>224</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D57" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F57" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>236</v>
+        <v>225</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D58" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F58" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>237</v>
+        <v>226</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D59" s="1" t="s">
-        <v>364</v>
+        <v>353</v>
       </c>
       <c r="E59" s="1" t="s">
-        <v>238</v>
+        <v>227</v>
       </c>
       <c r="F59" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>239</v>
+        <v>228</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D60" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F60" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>240</v>
+        <v>229</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D61" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F61" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>241</v>
+        <v>230</v>
       </c>
       <c r="C62" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D62" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D62" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E62" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F62" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>242</v>
+        <v>231</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D63" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F63" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>243</v>
+        <v>232</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D64" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F64" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
       <c r="B65" s="1" t="s">
-        <v>244</v>
+        <v>233</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D65" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F65" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>245</v>
+        <v>234</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D66" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F66" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>246</v>
+        <v>235</v>
       </c>
       <c r="C67" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D67" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D67" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E67" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F67" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>247</v>
+        <v>236</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D68" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F68" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>248</v>
+        <v>237</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D69" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F69" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>249</v>
+        <v>238</v>
       </c>
       <c r="C70" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D70" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D70" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E70" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F70" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>250</v>
+        <v>239</v>
       </c>
       <c r="C71" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D71" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D71" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E71" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F71" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>251</v>
+        <v>240</v>
       </c>
       <c r="C72" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D72" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D72" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E72" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F72" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>252</v>
+        <v>241</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D73" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F73" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>253</v>
+        <v>242</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D74" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F74" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>254</v>
+        <v>243</v>
       </c>
       <c r="C75" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D75" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D75" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E75" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F75" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
       <c r="B76" s="1" t="s">
-        <v>255</v>
+        <v>244</v>
       </c>
       <c r="C76" s="1" t="s">
+        <v>340</v>
+      </c>
+      <c r="D76" s="1" t="s">
         <v>351</v>
       </c>
-      <c r="D76" s="1" t="s">
-        <v>362</v>
-      </c>
       <c r="E76" s="1" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="F76" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>256</v>
+        <v>245</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D77" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F77" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>257</v>
+        <v>246</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D78" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F78" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>258</v>
+        <v>247</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D79" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F79" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>259</v>
+        <v>248</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D80" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F80" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>260</v>
+        <v>249</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D81" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F81" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>261</v>
+        <v>250</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D82" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F82" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>262</v>
+        <v>251</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D83" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F83" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>263</v>
+        <v>252</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D84" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F84" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>264</v>
+        <v>253</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D85" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F85" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>265</v>
+        <v>254</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D86" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F86" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>266</v>
+        <v>255</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D87" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F87" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>267</v>
+        <v>256</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D88" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F88" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>268</v>
+        <v>257</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D89" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F89" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>269</v>
+        <v>258</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D90" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F90" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
       <c r="B91" s="1" t="s">
-        <v>270</v>
+        <v>259</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D91" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F91" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>271</v>
+        <v>260</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D92" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F92" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>272</v>
+        <v>261</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D93" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F93" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>273</v>
+        <v>262</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D94" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F94" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>274</v>
+        <v>263</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D95" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F95" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>275</v>
+        <v>264</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D96" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F96" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>276</v>
+        <v>265</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D97" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F97" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>277</v>
+        <v>266</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D98" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F98" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>279</v>
+        <v>268</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D99" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="E99" s="1" t="s">
-        <v>346</v>
+        <v>335</v>
       </c>
       <c r="F99" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>278</v>
+        <v>267</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D100" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="E100" s="1" t="s">
-        <v>347</v>
+        <v>336</v>
       </c>
       <c r="F100" s="1" t="s">
-        <v>360</v>
-      </c>
-    </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+        <v>349</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>280</v>
+        <v>269</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D101" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F101" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>281</v>
+        <v>270</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D102" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F102" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>282</v>
+        <v>271</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="D103" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F103" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>283</v>
+        <v>272</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D104" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F104" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>284</v>
+        <v>273</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D105" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F105" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>285</v>
+        <v>274</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D106" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="F106" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>286</v>
+        <v>275</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D107" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F107" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>287</v>
+        <v>276</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D108" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F108" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>288</v>
+        <v>277</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D109" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F109" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>289</v>
+        <v>278</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D110" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F110" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>290</v>
+        <v>279</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D111" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F111" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>291</v>
+        <v>280</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D112" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F112" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>292</v>
+        <v>281</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D113" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F113" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>293</v>
+        <v>282</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D114" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F114" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>294</v>
+        <v>283</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D115" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F115" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>295</v>
+        <v>284</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D116" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F116" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>296</v>
+        <v>285</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D117" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F117" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>297</v>
+        <v>286</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D118" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F118" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>298</v>
+        <v>287</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D119" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F119" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>299</v>
+        <v>288</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D120" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F120" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>300</v>
+        <v>289</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D121" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F121" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>301</v>
+        <v>290</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D122" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F122" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>302</v>
+        <v>291</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D123" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F123" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>303</v>
+        <v>292</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D124" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F124" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>304</v>
+        <v>293</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D125" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F125" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>305</v>
+        <v>294</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D126" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F126" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>306</v>
+        <v>295</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D127" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F127" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>307</v>
+        <v>296</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D128" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F128" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>308</v>
+        <v>297</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D129" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F129" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>309</v>
+        <v>298</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D130" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F130" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>310</v>
+        <v>299</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D131" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F131" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>311</v>
+        <v>300</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D132" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F132" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>312</v>
+        <v>301</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D133" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F133" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>313</v>
+        <v>302</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D134" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F134" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>314</v>
+        <v>303</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D135" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F135" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>315</v>
+        <v>304</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D136" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F136" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>316</v>
+        <v>305</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D137" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F137" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>317</v>
+        <v>306</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D138" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F138" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>318</v>
+        <v>307</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D139" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F139" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>319</v>
+        <v>308</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D140" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F140" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>320</v>
+        <v>309</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D141" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F141" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>321</v>
+        <v>310</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D142" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F142" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>322</v>
+        <v>311</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D143" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F143" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>323</v>
+        <v>312</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D144" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F144" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>324</v>
+        <v>313</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D145" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F145" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>325</v>
+        <v>314</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D146" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F146" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>326</v>
+        <v>315</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D147" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F147" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>327</v>
+        <v>316</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D148" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F148" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>328</v>
+        <v>317</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D149" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F149" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>329</v>
+        <v>318</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D150" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F150" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>330</v>
+        <v>319</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D151" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F151" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>331</v>
+        <v>320</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D152" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F152" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>332</v>
+        <v>321</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D153" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F153" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>333</v>
+        <v>322</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D154" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F154" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>334</v>
+        <v>323</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D155" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F155" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>335</v>
+        <v>324</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D156" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F156" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>336</v>
+        <v>325</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D157" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F157" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>337</v>
+        <v>326</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D158" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F158" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>338</v>
+        <v>327</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D159" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F159" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>339</v>
+        <v>328</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D160" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F160" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>340</v>
+        <v>329</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D161" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F161" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>341</v>
+        <v>330</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D162" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F162" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>342</v>
+        <v>331</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D163" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F163" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>343</v>
+        <v>332</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D164" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F164" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>344</v>
+        <v>333</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D165" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F165" s="1" t="s">
-        <v>358</v>
-      </c>
-    </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+        <v>347</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>345</v>
+        <v>334</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>351</v>
+        <v>340</v>
       </c>
       <c r="D166" s="1" t="s">
-        <v>350</v>
+        <v>339</v>
       </c>
       <c r="F166" s="1" t="s">
-        <v>358</v>
+        <v>347</v>
       </c>
     </row>
   </sheetData>
@@ -4452,25 +4840,292 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F7735-F42E-498C-BEC1-50736A9A963F}">
+  <dimension ref="B2:B17"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.88671875" style="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="4" t="s">
+        <v>358</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>359</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>361</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>362</v>
+      </c>
+    </row>
+    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
+        <v>363</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
+        <v>364</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>365</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
+        <v>366</v>
+      </c>
+    </row>
+    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
+        <v>367</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
+        <v>368</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B15" s="2" t="s">
+        <v>369</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
+        <v>370</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
+  <dimension ref="B2:C17"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.77734375" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>372</v>
+      </c>
+      <c r="C2" s="4"/>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>373</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>374</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>375</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>376</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>377</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
+        <v>378</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>379</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
+        <v>380</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
+        <v>381</v>
+      </c>
+    </row>
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
+        <v>382</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B15" s="1" t="s">
+        <v>383</v>
+      </c>
+    </row>
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
-  <dimension ref="A1"/>
-  <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <dimension ref="B2:B16"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.77734375" style="1"/>
   </cols>
-  <sheetData/>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>386</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>389</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>390</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
+        <v>391</v>
+      </c>
+    </row>
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
+        <v>392</v>
+      </c>
+    </row>
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
+        <v>393</v>
+      </c>
+    </row>
+    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
+        <v>394</v>
+      </c>
+    </row>
+    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B13" s="2" t="s">
+        <v>395</v>
+      </c>
+    </row>
+    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B15" s="1" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BB7FF8-2BA0-4E37-9F78-C30173234A80}">
+  <dimension ref="B2:B6"/>
+  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <cols>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.88671875" style="1"/>
+  </cols>
+  <sheetData>
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B2" s="2" t="s">
+        <v>399</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>400</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
+        <v>403</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
effettuata la conversione nei dtypes corretti nel notebook ipynb
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C7049A00-E799-4FA5-BB81-B16E4B5CE4D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6F081E-305E-4296-9FDA-C22781FD37C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" activeTab="4" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="860" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -1945,7 +1945,7 @@
     <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="17.109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5546875" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
     <col min="7" max="16384" width="8.77734375" style="1"/>

</xml_diff>

<commit_message>
risposto alle prime due domande con creazione di relativi grafici
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF6F081E-305E-4296-9FDA-C22781FD37C5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA861492-B01D-4999-9A52-3A1DBDDE4B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="860" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -51,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="896" uniqueCount="404">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -1537,6 +1537,9 @@
       </rPr>
       <t>?</t>
     </r>
+  </si>
+  <si>
+    <t>FATTO</t>
   </si>
 </sst>
 </file>
@@ -4841,7 +4844,7 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F7735-F42E-498C-BEC1-50736A9A963F}">
-  <dimension ref="B2:B17"/>
+  <dimension ref="B2:C17"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
@@ -4849,67 +4852,73 @@
     <col min="3" max="16384" width="8.88671875" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="4" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>359</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="C3" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>360</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="C4" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>361</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="7" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>370</v>
       </c>

</xml_diff>

<commit_message>
completata la domanda sulla variabilità di durata delle partite
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FA861492-B01D-4999-9A52-3A1DBDDE4B8F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D58073-560A-E644-90DF-7DA08537B093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -51,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="898" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -1602,12 +1599,11 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1943,18 +1939,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5546875" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.77734375" style="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1974,7 +1970,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1991,7 +1987,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -2008,7 +2004,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -2025,7 +2021,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2045,7 +2041,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2062,7 +2058,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2079,7 +2075,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -2096,7 +2092,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2113,7 +2109,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -2133,7 +2129,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -2150,7 +2146,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -2170,7 +2166,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -2187,7 +2183,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -2204,7 +2200,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -2221,7 +2217,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -2238,7 +2234,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -2255,7 +2251,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -2272,7 +2268,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -2289,7 +2285,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -2306,7 +2302,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -2323,7 +2319,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -2340,7 +2336,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -2357,7 +2353,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -2374,7 +2370,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -2391,7 +2387,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -2408,7 +2404,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -2425,7 +2421,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -2442,7 +2438,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -2459,7 +2455,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -2476,7 +2472,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2493,7 +2489,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2510,7 +2506,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2527,7 +2523,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2544,7 +2540,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2561,7 +2557,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2578,7 +2574,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2595,7 +2591,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
@@ -2612,7 +2608,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -2629,7 +2625,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
@@ -2646,7 +2642,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
@@ -2663,7 +2659,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2683,7 +2679,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
@@ -2703,7 +2699,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -2723,7 +2719,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
@@ -2743,7 +2739,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -2760,7 +2756,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -2780,7 +2776,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -2800,7 +2796,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -2817,7 +2813,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -2834,7 +2830,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
@@ -2851,7 +2847,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
@@ -2868,7 +2864,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
@@ -2885,7 +2881,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
@@ -2902,7 +2898,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -2919,7 +2915,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -2936,7 +2932,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
@@ -2953,7 +2949,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
@@ -2970,7 +2966,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -2990,7 +2986,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -3007,7 +3003,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
@@ -3024,7 +3020,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -3044,7 +3040,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -3061,7 +3057,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
@@ -3078,7 +3074,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
@@ -3095,7 +3091,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
@@ -3112,7 +3108,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
@@ -3132,7 +3128,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
@@ -3149,7 +3145,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
@@ -3166,7 +3162,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
@@ -3186,7 +3182,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
@@ -3206,7 +3202,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
@@ -3226,7 +3222,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
@@ -3243,7 +3239,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
@@ -3260,7 +3256,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
@@ -3280,7 +3276,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
@@ -3300,7 +3296,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -3317,7 +3313,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
@@ -3334,7 +3330,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
@@ -3351,7 +3347,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
@@ -3368,7 +3364,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
@@ -3385,7 +3381,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
@@ -3402,7 +3398,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
@@ -3419,7 +3415,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -3436,7 +3432,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
@@ -3453,7 +3449,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
@@ -3470,7 +3466,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
@@ -3487,7 +3483,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
@@ -3504,7 +3500,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
@@ -3521,7 +3517,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
@@ -3538,7 +3534,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
@@ -3555,7 +3551,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
@@ -3572,7 +3568,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
@@ -3589,7 +3585,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
@@ -3606,7 +3602,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
@@ -3623,7 +3619,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
@@ -3640,7 +3636,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
@@ -3657,7 +3653,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
@@ -3674,7 +3670,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
@@ -3694,7 +3690,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
@@ -3714,7 +3710,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
@@ -3731,7 +3727,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
@@ -3748,7 +3744,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3765,7 +3761,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
@@ -3782,7 +3778,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
@@ -3799,7 +3795,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
@@ -3816,7 +3812,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
@@ -3833,7 +3829,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
@@ -3850,7 +3846,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
@@ -3867,7 +3863,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
@@ -3884,7 +3880,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
@@ -3901,7 +3897,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
@@ -3918,7 +3914,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
@@ -3935,7 +3931,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
@@ -3952,7 +3948,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
@@ -3969,7 +3965,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
@@ -3986,7 +3982,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
@@ -4003,7 +3999,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
@@ -4020,7 +4016,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -4037,7 +4033,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -4054,7 +4050,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
@@ -4071,7 +4067,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
@@ -4088,7 +4084,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
@@ -4105,7 +4101,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
@@ -4122,7 +4118,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
@@ -4139,7 +4135,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
@@ -4156,7 +4152,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
@@ -4173,7 +4169,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
@@ -4190,7 +4186,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
@@ -4207,7 +4203,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
@@ -4224,7 +4220,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
@@ -4241,7 +4237,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
@@ -4258,7 +4254,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
@@ -4275,7 +4271,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
@@ -4292,7 +4288,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
@@ -4309,7 +4305,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
@@ -4326,7 +4322,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
@@ -4343,7 +4339,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
@@ -4360,7 +4356,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
@@ -4377,7 +4373,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
@@ -4394,7 +4390,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
@@ -4411,7 +4407,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
@@ -4428,7 +4424,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
@@ -4445,7 +4441,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
@@ -4462,7 +4458,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
@@ -4479,7 +4475,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -4496,7 +4492,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
@@ -4513,7 +4509,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
@@ -4530,7 +4526,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
@@ -4547,7 +4543,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
@@ -4564,7 +4560,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
@@ -4581,7 +4577,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
@@ -4598,7 +4594,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
@@ -4615,7 +4611,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
@@ -4632,7 +4628,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
@@ -4649,7 +4645,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -4666,7 +4662,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
@@ -4683,7 +4679,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
@@ -4700,7 +4696,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
@@ -4717,7 +4713,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
@@ -4734,7 +4730,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
@@ -4751,7 +4747,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
@@ -4768,7 +4764,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
@@ -4785,7 +4781,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
@@ -4802,7 +4798,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
@@ -4819,7 +4815,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
@@ -4845,19 +4841,19 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F7735-F42E-498C-BEC1-50736A9A963F}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
-      <c r="B2" s="4" t="s">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B2" s="2" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>359</v>
       </c>
@@ -4865,7 +4861,7 @@
         <v>404</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>360</v>
       </c>
@@ -4873,57 +4869,60 @@
         <v>404</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>361</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C5" s="1" t="s">
+        <v>404</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="2" t="s">
         <v>369</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>370</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>371</v>
       </c>
@@ -4936,80 +4935,80 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>372</v>
       </c>
-      <c r="C2" s="4"/>
-    </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>383</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>385</v>
       </c>
@@ -5022,74 +5021,74 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
   <dimension ref="B2:B16"/>
-  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
         <v>396</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>398</v>
       </c>
@@ -5102,34 +5101,34 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BB7FF8-2BA0-4E37-9F78-C30173234A80}">
   <dimension ref="B2:B6"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.88671875" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>401</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>403</v>
       </c>

</xml_diff>

<commit_message>
risposto alle ultime due domande delle analisi generali
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10125"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D0D58073-560A-E644-90DF-7DA08537B093}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4DA4A2-3812-4AC5-B048-B212197E1D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -48,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="899" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -1134,35 +1137,6 @@
   </si>
   <si>
     <t>La durata media delle partite LEC  è variata nei vari split??</t>
-  </si>
-  <si>
-    <r>
-      <t>Qual è la percentuale di vittorie BLUE SIDE</t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t xml:space="preserve"> </t>
-    </r>
-    <r>
-      <rPr>
-        <sz val="11"/>
-        <color theme="1"/>
-        <rFont val="Aptos Narrow"/>
-        <family val="2"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>vs RED SIDE nel LEC 2025?</t>
-    </r>
-  </si>
-  <si>
-    <t>Esiste una correlazione tra durata della partita e probabilità di vittoria?</t>
   </si>
   <si>
     <t>Meta &amp; ritmo di gioco</t>
@@ -1537,6 +1511,12 @@
   </si>
   <si>
     <t>FATTO</t>
+  </si>
+  <si>
+    <t>la percentuale delle vittorie di un side viene influenzata dalla lunghezza della partita?</t>
+  </si>
+  <si>
+    <t>la percentuale di vittorie Blue side vs red side varia tra i vari split?</t>
   </si>
 </sst>
 </file>
@@ -1939,18 +1919,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="1"/>
+    <col min="7" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1970,7 +1950,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1987,7 +1967,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -2004,7 +1984,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -2021,7 +2001,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2041,7 +2021,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2058,7 +2038,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2075,7 +2055,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -2092,7 +2072,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2109,7 +2089,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -2129,7 +2109,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -2146,7 +2126,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -2166,7 +2146,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -2183,7 +2163,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -2200,7 +2180,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -2217,7 +2197,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -2234,7 +2214,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -2251,7 +2231,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -2268,7 +2248,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -2285,7 +2265,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -2302,7 +2282,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -2319,7 +2299,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -2336,7 +2316,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -2353,7 +2333,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -2370,7 +2350,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -2387,7 +2367,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -2404,7 +2384,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -2421,7 +2401,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -2438,7 +2418,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -2455,7 +2435,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -2472,7 +2452,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2489,7 +2469,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2506,7 +2486,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2523,7 +2503,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2540,7 +2520,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2557,7 +2537,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2574,7 +2554,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2591,7 +2571,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
@@ -2608,7 +2588,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -2625,7 +2605,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
@@ -2642,7 +2622,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
@@ -2659,7 +2639,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2679,7 +2659,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
@@ -2699,7 +2679,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -2719,7 +2699,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
@@ -2739,7 +2719,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -2756,7 +2736,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -2776,7 +2756,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -2796,7 +2776,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -2813,7 +2793,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -2830,7 +2810,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
@@ -2847,7 +2827,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
@@ -2864,7 +2844,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
@@ -2881,7 +2861,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
@@ -2898,7 +2878,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -2915,7 +2895,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -2932,7 +2912,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
@@ -2949,7 +2929,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
@@ -2966,7 +2946,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -2986,7 +2966,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -3003,7 +2983,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
@@ -3020,7 +3000,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -3040,7 +3020,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -3057,7 +3037,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
@@ -3074,7 +3054,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
@@ -3091,7 +3071,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
@@ -3108,7 +3088,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
@@ -3128,7 +3108,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
@@ -3145,7 +3125,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
@@ -3162,7 +3142,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
@@ -3182,7 +3162,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
@@ -3202,7 +3182,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
@@ -3222,7 +3202,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
@@ -3239,7 +3219,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
@@ -3256,7 +3236,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
@@ -3276,7 +3256,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
@@ -3296,7 +3276,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -3313,7 +3293,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
@@ -3330,7 +3310,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
@@ -3347,7 +3327,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
@@ -3364,7 +3344,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
@@ -3381,7 +3361,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
@@ -3398,7 +3378,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
@@ -3415,7 +3395,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -3432,7 +3412,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
@@ -3449,7 +3429,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
@@ -3466,7 +3446,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
@@ -3483,7 +3463,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
@@ -3500,7 +3480,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
@@ -3517,7 +3497,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
@@ -3534,7 +3514,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
@@ -3551,7 +3531,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
@@ -3568,7 +3548,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
@@ -3585,7 +3565,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
@@ -3602,7 +3582,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
@@ -3619,7 +3599,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
@@ -3636,7 +3616,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
@@ -3653,7 +3633,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
@@ -3670,7 +3650,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
@@ -3690,7 +3670,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
@@ -3710,7 +3690,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
@@ -3727,7 +3707,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
@@ -3744,7 +3724,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3761,7 +3741,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
@@ -3778,7 +3758,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
@@ -3795,7 +3775,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
@@ -3812,7 +3792,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
@@ -3829,7 +3809,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
@@ -3846,7 +3826,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
@@ -3863,7 +3843,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
@@ -3880,7 +3860,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
@@ -3897,7 +3877,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
@@ -3914,7 +3894,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
@@ -3931,7 +3911,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
@@ -3948,7 +3928,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
@@ -3965,7 +3945,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
@@ -3982,7 +3962,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
@@ -3999,7 +3979,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
@@ -4016,7 +3996,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -4033,7 +4013,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -4050,7 +4030,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
@@ -4067,7 +4047,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
@@ -4084,7 +4064,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
@@ -4101,7 +4081,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
@@ -4118,7 +4098,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
@@ -4135,7 +4115,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
@@ -4152,7 +4132,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
@@ -4169,7 +4149,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
@@ -4186,7 +4166,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
@@ -4203,7 +4183,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
@@ -4220,7 +4200,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
@@ -4237,7 +4217,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
@@ -4254,7 +4234,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
@@ -4271,7 +4251,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
@@ -4288,7 +4268,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
@@ -4305,7 +4285,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
@@ -4322,7 +4302,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
@@ -4339,7 +4319,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
@@ -4356,7 +4336,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
@@ -4373,7 +4353,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
@@ -4390,7 +4370,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
@@ -4407,7 +4387,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
@@ -4424,7 +4404,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
@@ -4441,7 +4421,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
@@ -4458,7 +4438,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
@@ -4475,7 +4455,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -4492,7 +4472,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
@@ -4509,7 +4489,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
@@ -4526,7 +4506,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
@@ -4543,7 +4523,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
@@ -4560,7 +4540,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
@@ -4577,7 +4557,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
@@ -4594,7 +4574,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
@@ -4611,7 +4591,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
@@ -4628,7 +4608,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
@@ -4645,7 +4625,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -4662,7 +4642,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
@@ -4679,7 +4659,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
@@ -4696,7 +4676,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
@@ -4713,7 +4693,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
@@ -4730,7 +4710,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
@@ -4747,7 +4727,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
@@ -4764,7 +4744,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
@@ -4781,7 +4761,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
@@ -4798,7 +4778,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
@@ -4815,7 +4795,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
@@ -4841,90 +4821,98 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F7735-F42E-498C-BEC1-50736A9A963F}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" style="1"/>
+    <col min="4" max="4" width="49.88671875" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>359</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>360</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>404</v>
-      </c>
-    </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>361</v>
       </c>
       <c r="C5" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
         <v>404</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B6" s="1" t="s">
+      <c r="C6" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B7" s="1" t="s">
+        <v>403</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B9" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B7" s="1" t="s">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
         <v>363</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B9" s="2" t="s">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
         <v>364</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B10" s="1" t="s">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
         <v>365</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B13" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B15" s="2" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B13" s="1" t="s">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
         <v>368</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B15" s="2" t="s">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
         <v>369</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B16" s="1" t="s">
-        <v>370</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B17" s="1" t="s">
-        <v>371</v>
       </c>
     </row>
   </sheetData>
@@ -4935,82 +4923,82 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
+        <v>370</v>
+      </c>
+      <c r="C2" s="2"/>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>371</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
         <v>372</v>
       </c>
-      <c r="C2" s="2"/>
-    </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B4" s="1" t="s">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B5" s="1" t="s">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B6" s="1" t="s">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B8" s="2" t="s">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B10" s="1" t="s">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B12" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B14" s="2" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B12" s="1" t="s">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B15" s="1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B14" s="2" t="s">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="s">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B17" s="1" t="s">
         <v>383</v>
-      </c>
-    </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
-      <c r="B16" s="1" t="s">
-        <v>384</v>
-      </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B17" s="1" t="s">
-        <v>385</v>
       </c>
     </row>
   </sheetData>
@@ -5021,76 +5009,76 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
   <dimension ref="B2:B16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
+        <v>384</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>387</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
+        <v>385</v>
+      </c>
+    </row>
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
+        <v>388</v>
+      </c>
+    </row>
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B8" s="2" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B4" s="1" t="s">
-        <v>387</v>
-      </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B5" s="1" t="s">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B9" s="1" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B6" s="1" t="s">
-        <v>388</v>
-      </c>
-    </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B8" s="2" t="s">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B10" s="1" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B9" s="1" t="s">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B11" s="1" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B10" s="1" t="s">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B13" s="2" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B11" s="1" t="s">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B14" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B13" s="2" t="s">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B15" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B14" s="1" t="s">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B16" s="1" t="s">
         <v>396</v>
-      </c>
-    </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B15" s="1" t="s">
-        <v>397</v>
-      </c>
-    </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B16" s="1" t="s">
-        <v>398</v>
       </c>
     </row>
   </sheetData>
@@ -5101,36 +5089,36 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BB7FF8-2BA0-4E37-9F78-C30173234A80}">
   <dimension ref="B2:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
+        <v>397</v>
+      </c>
+    </row>
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B3" s="1" t="s">
+        <v>398</v>
+      </c>
+    </row>
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B4" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B5" s="1" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B4" s="1" t="s">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="B6" s="1" t="s">
         <v>401</v>
-      </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B5" s="1" t="s">
-        <v>402</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B6" s="1" t="s">
-        <v>403</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
terminata la fase di analisi generale
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A4DA4A2-3812-4AC5-B048-B212197E1D05}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F785914F-BC27-3E43-A87D-5C480AEAC0DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -51,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="901" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -1919,18 +1916,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.77734375" style="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1950,7 +1947,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1967,7 +1964,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1984,7 +1981,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -2001,7 +1998,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2021,7 +2018,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2038,7 +2035,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2055,7 +2052,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -2072,7 +2069,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2089,7 +2086,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -2109,7 +2106,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -2126,7 +2123,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -2146,7 +2143,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -2163,7 +2160,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -2180,7 +2177,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -2197,7 +2194,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -2214,7 +2211,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -2231,7 +2228,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -2248,7 +2245,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -2265,7 +2262,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -2282,7 +2279,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -2299,7 +2296,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -2316,7 +2313,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -2333,7 +2330,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -2350,7 +2347,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -2367,7 +2364,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -2384,7 +2381,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -2401,7 +2398,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -2418,7 +2415,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -2435,7 +2432,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -2452,7 +2449,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2469,7 +2466,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2486,7 +2483,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2503,7 +2500,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2520,7 +2517,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2537,7 +2534,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2554,7 +2551,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2571,7 +2568,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
@@ -2588,7 +2585,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -2605,7 +2602,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
@@ -2622,7 +2619,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
@@ -2639,7 +2636,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2659,7 +2656,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
@@ -2679,7 +2676,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -2699,7 +2696,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
@@ -2719,7 +2716,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -2736,7 +2733,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -2756,7 +2753,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -2776,7 +2773,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -2793,7 +2790,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -2810,7 +2807,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
@@ -2827,7 +2824,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
@@ -2844,7 +2841,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
@@ -2861,7 +2858,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
@@ -2878,7 +2875,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -2895,7 +2892,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -2912,7 +2909,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
@@ -2929,7 +2926,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
@@ -2946,7 +2943,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -2966,7 +2963,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -2983,7 +2980,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
@@ -3000,7 +2997,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -3020,7 +3017,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -3037,7 +3034,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
@@ -3054,7 +3051,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
@@ -3071,7 +3068,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
@@ -3088,7 +3085,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
@@ -3108,7 +3105,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
@@ -3125,7 +3122,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
@@ -3142,7 +3139,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
@@ -3162,7 +3159,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
@@ -3182,7 +3179,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
@@ -3202,7 +3199,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
@@ -3219,7 +3216,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
@@ -3236,7 +3233,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
@@ -3256,7 +3253,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
@@ -3276,7 +3273,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -3293,7 +3290,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
@@ -3310,7 +3307,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
@@ -3327,7 +3324,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
@@ -3344,7 +3341,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
@@ -3361,7 +3358,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
@@ -3378,7 +3375,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
@@ -3395,7 +3392,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -3412,7 +3409,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
@@ -3429,7 +3426,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
@@ -3446,7 +3443,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
@@ -3463,7 +3460,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
@@ -3480,7 +3477,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
@@ -3497,7 +3494,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
@@ -3514,7 +3511,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
@@ -3531,7 +3528,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
@@ -3548,7 +3545,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
@@ -3565,7 +3562,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
@@ -3582,7 +3579,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
@@ -3599,7 +3596,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
@@ -3616,7 +3613,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
@@ -3633,7 +3630,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
@@ -3650,7 +3647,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
@@ -3670,7 +3667,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
@@ -3690,7 +3687,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
@@ -3707,7 +3704,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
@@ -3724,7 +3721,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3741,7 +3738,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
@@ -3758,7 +3755,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
@@ -3775,7 +3772,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
@@ -3792,7 +3789,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
@@ -3809,7 +3806,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
@@ -3826,7 +3823,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
@@ -3843,7 +3840,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
@@ -3860,7 +3857,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
@@ -3877,7 +3874,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
@@ -3894,7 +3891,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
@@ -3911,7 +3908,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
@@ -3928,7 +3925,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
@@ -3945,7 +3942,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
@@ -3962,7 +3959,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
@@ -3979,7 +3976,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
@@ -3996,7 +3993,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -4013,7 +4010,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -4030,7 +4027,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
@@ -4047,7 +4044,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
@@ -4064,7 +4061,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
@@ -4081,7 +4078,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
@@ -4098,7 +4095,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
@@ -4115,7 +4112,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
@@ -4132,7 +4129,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
@@ -4149,7 +4146,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
@@ -4166,7 +4163,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
@@ -4183,7 +4180,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
@@ -4200,7 +4197,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
@@ -4217,7 +4214,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
@@ -4234,7 +4231,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
@@ -4251,7 +4248,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
@@ -4268,7 +4265,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
@@ -4285,7 +4282,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
@@ -4302,7 +4299,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
@@ -4319,7 +4316,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
@@ -4336,7 +4333,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
@@ -4353,7 +4350,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
@@ -4370,7 +4367,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
@@ -4387,7 +4384,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
@@ -4404,7 +4401,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
@@ -4421,7 +4418,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
@@ -4438,7 +4435,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
@@ -4455,7 +4452,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -4472,7 +4469,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
@@ -4489,7 +4486,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
@@ -4506,7 +4503,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
@@ -4523,7 +4520,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
@@ -4540,7 +4537,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
@@ -4557,7 +4554,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
@@ -4574,7 +4571,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
@@ -4591,7 +4588,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
@@ -4608,7 +4605,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
@@ -4625,7 +4622,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -4642,7 +4639,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
@@ -4659,7 +4656,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
@@ -4676,7 +4673,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
@@ -4693,7 +4690,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
@@ -4710,7 +4707,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
@@ -4727,7 +4724,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
@@ -4744,7 +4741,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
@@ -4761,7 +4758,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
@@ -4778,7 +4775,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
@@ -4795,7 +4792,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
@@ -4821,21 +4818,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F7735-F42E-498C-BEC1-50736A9A963F}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.77734375" style="1"/>
-    <col min="4" max="4" width="49.88671875" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" style="1"/>
+    <col min="4" max="4" width="49.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>359</v>
       </c>
@@ -4843,7 +4840,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>360</v>
       </c>
@@ -4851,7 +4848,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>361</v>
       </c>
@@ -4859,7 +4856,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>404</v>
       </c>
@@ -4867,7 +4864,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
         <v>403</v>
       </c>
@@ -4875,44 +4872,59 @@
         <v>402</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>363</v>
       </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C10" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>364</v>
       </c>
-    </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C11" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>365</v>
       </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C12" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="2" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>368</v>
       </c>
-    </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+      <c r="C16" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>369</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -4923,80 +4935,80 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>370</v>
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>371</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>372</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>373</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>374</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>376</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>377</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>378</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>379</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>381</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>382</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>383</v>
       </c>
@@ -5009,74 +5021,74 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
   <dimension ref="B2:B16"/>
-  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>387</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>385</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>396</v>
       </c>
@@ -5089,34 +5101,34 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BB7FF8-2BA0-4E37-9F78-C30173234A80}">
   <dimension ref="B2:B6"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>401</v>
       </c>

</xml_diff>

<commit_message>
effettuata analisi delle prime due domande relative alle performance di team
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F785914F-BC27-3E43-A87D-5C480AEAC0DF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32C73F7-5693-4448-8404-577AD69D926D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="1" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="2" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="906" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -4952,10 +4952,16 @@
       <c r="B3" s="1" t="s">
         <v>371</v>
       </c>
+      <c r="C3" s="1" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>372</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
completate domande sotto gruppo uno delle performance di team
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B32C73F7-5693-4448-8404-577AD69D926D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0A4728-D101-954B-AEA2-9FEDDA460A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="2" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="908" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -4968,10 +4968,16 @@
       <c r="B5" s="1" t="s">
         <v>373</v>
       </c>
+      <c r="C5" s="1" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>374</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
portato avanti lo studio sulle analisi di team, mancante solo l'ultima domanda2 git push
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10201"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5D0A4728-D101-954B-AEA2-9FEDDA460A32}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39D777B-01F1-B94F-8AAC-489C1CE5FD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="2" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="910" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -4989,21 +4989,33 @@
       <c r="B9" s="1" t="s">
         <v>376</v>
       </c>
+      <c r="C9" s="1" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>377</v>
       </c>
+      <c r="C10" s="1" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>378</v>
       </c>
+      <c r="C11" s="1" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>379</v>
       </c>
+      <c r="C12" s="1" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
@@ -5014,10 +5026,16 @@
       <c r="B15" s="1" t="s">
         <v>381</v>
       </c>
+      <c r="C15" s="1" t="s">
+        <v>402</v>
+      </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>382</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>402</v>
       </c>
     </row>
     <row r="17" spans="2:2" x14ac:dyDescent="0.2">

</xml_diff>

<commit_message>
iniziate analisi su performance individuali
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A39D777B-01F1-B94F-8AAC-489C1CE5FD6B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0758FB4A-0B75-E344-BD89-49CD128879C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="2" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="3" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="916" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -5038,9 +5038,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="17" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>383</v>
+      </c>
+      <c r="C17" s="1" t="s">
+        <v>402</v>
       </c>
     </row>
   </sheetData>
@@ -5050,7 +5053,7 @@
 
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
-  <dimension ref="B2:B16"/>
+  <dimension ref="B2:C16"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
@@ -5058,67 +5061,73 @@
     <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>387</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="C3" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>385</v>
       </c>
-    </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+      <c r="C4" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>388</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>386</v>
       </c>
     </row>
-    <row r="8" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="9" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>390</v>
       </c>
     </row>
-    <row r="10" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>391</v>
       </c>
     </row>
-    <row r="11" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>392</v>
       </c>
     </row>
-    <row r="13" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="14" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="15" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="16" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>396</v>
       </c>

</xml_diff>

<commit_message>
fatte le prime due sezioni delle analisi individuali
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0758FB4A-0B75-E344-BD89-49CD128879C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BD3755-5E90-450F-ACFD-CCEBFCF2A663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="3" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="860" activeTab="3" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -35,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -48,7 +51,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="919" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -1916,18 +1919,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.5" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.44140625" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.83203125" style="1"/>
+    <col min="7" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1947,7 +1950,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1964,7 +1967,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1981,7 +1984,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -1998,7 +2001,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2018,7 +2021,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2035,7 +2038,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2052,7 +2055,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -2069,7 +2072,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2086,7 +2089,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -2106,7 +2109,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -2123,7 +2126,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -2143,7 +2146,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -2160,7 +2163,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -2177,7 +2180,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -2194,7 +2197,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -2211,7 +2214,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -2228,7 +2231,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -2245,7 +2248,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -2262,7 +2265,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -2279,7 +2282,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -2296,7 +2299,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -2313,7 +2316,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -2330,7 +2333,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -2347,7 +2350,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -2364,7 +2367,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -2381,7 +2384,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -2398,7 +2401,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -2415,7 +2418,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -2432,7 +2435,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -2449,7 +2452,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2466,7 +2469,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2483,7 +2486,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2500,7 +2503,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2517,7 +2520,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2534,7 +2537,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2551,7 +2554,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2568,7 +2571,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
@@ -2585,7 +2588,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -2602,7 +2605,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
@@ -2619,7 +2622,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
@@ -2636,7 +2639,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2656,7 +2659,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
@@ -2676,7 +2679,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -2696,7 +2699,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
@@ -2716,7 +2719,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -2733,7 +2736,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -2753,7 +2756,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -2773,7 +2776,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -2790,7 +2793,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -2807,7 +2810,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
@@ -2824,7 +2827,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
@@ -2841,7 +2844,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
@@ -2858,7 +2861,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
@@ -2875,7 +2878,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -2892,7 +2895,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -2909,7 +2912,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
@@ -2926,7 +2929,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
@@ -2943,7 +2946,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -2963,7 +2966,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -2980,7 +2983,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
@@ -2997,7 +3000,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -3017,7 +3020,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -3034,7 +3037,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
@@ -3051,7 +3054,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
@@ -3068,7 +3071,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
@@ -3085,7 +3088,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
@@ -3105,7 +3108,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
@@ -3122,7 +3125,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
@@ -3139,7 +3142,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
@@ -3159,7 +3162,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
@@ -3179,7 +3182,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
@@ -3199,7 +3202,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
@@ -3216,7 +3219,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
@@ -3233,7 +3236,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
@@ -3253,7 +3256,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
@@ -3273,7 +3276,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -3290,7 +3293,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
@@ -3307,7 +3310,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
@@ -3324,7 +3327,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
@@ -3341,7 +3344,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
@@ -3358,7 +3361,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
@@ -3375,7 +3378,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
@@ -3392,7 +3395,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -3409,7 +3412,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
@@ -3426,7 +3429,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
@@ -3443,7 +3446,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
@@ -3460,7 +3463,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
@@ -3477,7 +3480,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
@@ -3494,7 +3497,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
@@ -3511,7 +3514,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
@@ -3528,7 +3531,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
@@ -3545,7 +3548,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
@@ -3562,7 +3565,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
@@ -3579,7 +3582,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
@@ -3596,7 +3599,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
@@ -3613,7 +3616,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
@@ -3630,7 +3633,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
@@ -3647,7 +3650,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
@@ -3667,7 +3670,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
@@ -3687,7 +3690,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
@@ -3704,7 +3707,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
@@ -3721,7 +3724,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3738,7 +3741,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
@@ -3755,7 +3758,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
@@ -3772,7 +3775,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
@@ -3789,7 +3792,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
@@ -3806,7 +3809,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
@@ -3823,7 +3826,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
@@ -3840,7 +3843,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
@@ -3857,7 +3860,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
@@ -3874,7 +3877,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
@@ -3891,7 +3894,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
@@ -3908,7 +3911,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
@@ -3925,7 +3928,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
@@ -3942,7 +3945,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
@@ -3959,7 +3962,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
@@ -3976,7 +3979,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
@@ -3993,7 +3996,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -4010,7 +4013,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -4027,7 +4030,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
@@ -4044,7 +4047,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
@@ -4061,7 +4064,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
@@ -4078,7 +4081,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
@@ -4095,7 +4098,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
@@ -4112,7 +4115,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
@@ -4129,7 +4132,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
@@ -4146,7 +4149,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
@@ -4163,7 +4166,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
@@ -4180,7 +4183,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
@@ -4197,7 +4200,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
@@ -4214,7 +4217,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
@@ -4231,7 +4234,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
@@ -4248,7 +4251,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
@@ -4265,7 +4268,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
@@ -4282,7 +4285,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
@@ -4299,7 +4302,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
@@ -4316,7 +4319,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
@@ -4333,7 +4336,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
@@ -4350,7 +4353,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
@@ -4367,7 +4370,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
@@ -4384,7 +4387,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
@@ -4401,7 +4404,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
@@ -4418,7 +4421,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
@@ -4435,7 +4438,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
@@ -4452,7 +4455,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -4469,7 +4472,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
@@ -4486,7 +4489,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
@@ -4503,7 +4506,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
@@ -4520,7 +4523,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
@@ -4537,7 +4540,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
@@ -4554,7 +4557,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
@@ -4571,7 +4574,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
@@ -4588,7 +4591,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
@@ -4605,7 +4608,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
@@ -4622,7 +4625,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -4639,7 +4642,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
@@ -4656,7 +4659,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
@@ -4673,7 +4676,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
@@ -4690,7 +4693,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
@@ -4707,7 +4710,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
@@ -4724,7 +4727,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
@@ -4741,7 +4744,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
@@ -4758,7 +4761,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
@@ -4775,7 +4778,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
@@ -4792,7 +4795,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
@@ -4818,21 +4821,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F7735-F42E-498C-BEC1-50736A9A963F}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.83203125" style="1"/>
-    <col min="4" max="4" width="49.83203125" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.77734375" style="1"/>
+    <col min="4" max="4" width="49.77734375" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>359</v>
       </c>
@@ -4840,7 +4843,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>360</v>
       </c>
@@ -4848,7 +4851,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>361</v>
       </c>
@@ -4856,7 +4859,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>404</v>
       </c>
@@ -4864,7 +4867,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B7" s="1" t="s">
         <v>403</v>
       </c>
@@ -4872,12 +4875,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>363</v>
       </c>
@@ -4885,7 +4888,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>364</v>
       </c>
@@ -4893,7 +4896,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>365</v>
       </c>
@@ -4901,17 +4904,17 @@
         <v>402</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B13" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B15" s="2" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>368</v>
       </c>
@@ -4919,7 +4922,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>369</v>
       </c>
@@ -4935,20 +4938,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>370</v>
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>371</v>
       </c>
@@ -4956,7 +4959,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>372</v>
       </c>
@@ -4964,7 +4967,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>373</v>
       </c>
@@ -4972,7 +4975,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>374</v>
       </c>
@@ -4980,12 +4983,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>376</v>
       </c>
@@ -4993,7 +4996,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>377</v>
       </c>
@@ -5001,7 +5004,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>378</v>
       </c>
@@ -5009,7 +5012,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B12" s="1" t="s">
         <v>379</v>
       </c>
@@ -5017,12 +5020,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B14" s="2" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>381</v>
       </c>
@@ -5030,7 +5033,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>382</v>
       </c>
@@ -5038,7 +5041,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B17" s="1" t="s">
         <v>383</v>
       </c>
@@ -5054,19 +5057,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
   <dimension ref="B2:C16"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>387</v>
       </c>
@@ -5074,7 +5077,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>385</v>
       </c>
@@ -5082,52 +5085,67 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>388</v>
       </c>
-    </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C5" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>386</v>
       </c>
-    </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C6" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B8" s="2" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B9" s="1" t="s">
         <v>390</v>
       </c>
-    </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C9" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B10" s="1" t="s">
         <v>391</v>
       </c>
-    </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C10" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B11" s="1" t="s">
         <v>392</v>
       </c>
-    </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="C11" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B13" s="2" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B14" s="1" t="s">
         <v>394</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B15" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
       <c r="B16" s="1" t="s">
         <v>396</v>
       </c>
@@ -5140,34 +5158,34 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BB7FF8-2BA0-4E37-9F78-C30173234A80}">
   <dimension ref="B2:B6"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
+  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
-    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.83203125" style="1"/>
+    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.77734375" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B2" s="2" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B3" s="1" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B4" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B5" s="1" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
       <c r="B6" s="1" t="s">
         <v>401</v>
       </c>

</xml_diff>

<commit_message>
risposto alla domanda sulle stabilità delle performance
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27932"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10208"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\aless\Documents\data_analysis\G2-project-analysis\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{82BD3755-5E90-450F-ACFD-CCEBFCF2A663}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3422682-1BF7-724D-ADF6-8E56FBCCE6C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" tabRatio="860" activeTab="3" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="23260" windowHeight="12460" tabRatio="860" activeTab="3" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -35,9 +35,6 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
@@ -51,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="924" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -1919,18 +1916,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{F0051469-D03D-4184-AAF0-6F8CC0E4CC98}">
   <dimension ref="A1:F166"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="23.44140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="23.5" style="1" bestFit="1" customWidth="1"/>
     <col min="2" max="2" width="66.6640625" style="1" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="15" style="1" customWidth="1"/>
-    <col min="4" max="4" width="18.44140625" style="1" customWidth="1"/>
+    <col min="4" max="4" width="18.5" style="1" customWidth="1"/>
     <col min="5" max="5" width="50.33203125" style="1" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="27.6640625" style="1" customWidth="1"/>
-    <col min="7" max="16384" width="8.77734375" style="1"/>
+    <col min="7" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="1" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A1" s="2" t="s">
         <v>165</v>
       </c>
@@ -1950,7 +1947,7 @@
         <v>341</v>
       </c>
     </row>
-    <row r="2" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="2" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A2" s="1" t="s">
         <v>0</v>
       </c>
@@ -1967,7 +1964,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="3" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="3" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A3" s="1" t="s">
         <v>1</v>
       </c>
@@ -1984,7 +1981,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="4" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="4" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A4" s="1" t="s">
         <v>2</v>
       </c>
@@ -2001,7 +1998,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="5" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A5" s="1" t="s">
         <v>3</v>
       </c>
@@ -2021,7 +2018,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="6" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="6" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A6" s="1" t="s">
         <v>4</v>
       </c>
@@ -2038,7 +2035,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="7" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A7" s="1" t="s">
         <v>5</v>
       </c>
@@ -2055,7 +2052,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="8" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A8" s="1" t="s">
         <v>6</v>
       </c>
@@ -2072,7 +2069,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="9" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A9" s="1" t="s">
         <v>7</v>
       </c>
@@ -2089,7 +2086,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="10" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A10" s="1" t="s">
         <v>8</v>
       </c>
@@ -2109,7 +2106,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="11" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A11" s="1" t="s">
         <v>9</v>
       </c>
@@ -2126,7 +2123,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="12" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A12" s="1" t="s">
         <v>10</v>
       </c>
@@ -2146,7 +2143,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="13" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="13" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A13" s="1" t="s">
         <v>11</v>
       </c>
@@ -2163,7 +2160,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="14" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="14" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A14" s="1" t="s">
         <v>12</v>
       </c>
@@ -2180,7 +2177,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="15" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="15" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A15" s="1" t="s">
         <v>13</v>
       </c>
@@ -2197,7 +2194,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="16" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="16" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A16" s="1" t="s">
         <v>14</v>
       </c>
@@ -2214,7 +2211,7 @@
         <v>343</v>
       </c>
     </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="17" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A17" s="1" t="s">
         <v>15</v>
       </c>
@@ -2231,7 +2228,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="18" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A18" s="1" t="s">
         <v>16</v>
       </c>
@@ -2248,7 +2245,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="19" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A19" s="1" t="s">
         <v>17</v>
       </c>
@@ -2265,7 +2262,7 @@
         <v>344</v>
       </c>
     </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="20" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A20" s="1" t="s">
         <v>18</v>
       </c>
@@ -2282,7 +2279,7 @@
         <v>348</v>
       </c>
     </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="21" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A21" s="1" t="s">
         <v>19</v>
       </c>
@@ -2299,7 +2296,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="22" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A22" s="1" t="s">
         <v>20</v>
       </c>
@@ -2316,7 +2313,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="23" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A23" s="1" t="s">
         <v>21</v>
       </c>
@@ -2333,7 +2330,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="24" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A24" s="1" t="s">
         <v>22</v>
       </c>
@@ -2350,7 +2347,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="25" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A25" s="1" t="s">
         <v>23</v>
       </c>
@@ -2367,7 +2364,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="26" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A26" s="1" t="s">
         <v>24</v>
       </c>
@@ -2384,7 +2381,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="27" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A27" s="1" t="s">
         <v>25</v>
       </c>
@@ -2401,7 +2398,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="28" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A28" s="1" t="s">
         <v>26</v>
       </c>
@@ -2418,7 +2415,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="29" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A29" s="1" t="s">
         <v>27</v>
       </c>
@@ -2435,7 +2432,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="30" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A30" s="1" t="s">
         <v>28</v>
       </c>
@@ -2452,7 +2449,7 @@
         <v>346</v>
       </c>
     </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="31" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A31" s="1" t="s">
         <v>29</v>
       </c>
@@ -2469,7 +2466,7 @@
         <v>342</v>
       </c>
     </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="32" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A32" s="1" t="s">
         <v>30</v>
       </c>
@@ -2486,7 +2483,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="33" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="33" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A33" s="1" t="s">
         <v>31</v>
       </c>
@@ -2503,7 +2500,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="34" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="34" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A34" s="1" t="s">
         <v>32</v>
       </c>
@@ -2520,7 +2517,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="35" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="35" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A35" s="1" t="s">
         <v>33</v>
       </c>
@@ -2537,7 +2534,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="36" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="36" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A36" s="1" t="s">
         <v>34</v>
       </c>
@@ -2554,7 +2551,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="37" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="37" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A37" s="1" t="s">
         <v>35</v>
       </c>
@@ -2571,7 +2568,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="38" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="38" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A38" s="1" t="s">
         <v>36</v>
       </c>
@@ -2588,7 +2585,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="39" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="39" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A39" s="1" t="s">
         <v>37</v>
       </c>
@@ -2605,7 +2602,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="40" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="40" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A40" s="1" t="s">
         <v>38</v>
       </c>
@@ -2622,7 +2619,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="41" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="41" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A41" s="1" t="s">
         <v>39</v>
       </c>
@@ -2639,7 +2636,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="42" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="42" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A42" s="1" t="s">
         <v>40</v>
       </c>
@@ -2659,7 +2656,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="43" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="43" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A43" s="1" t="s">
         <v>41</v>
       </c>
@@ -2679,7 +2676,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="44" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="44" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A44" s="1" t="s">
         <v>42</v>
       </c>
@@ -2699,7 +2696,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="45" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="45" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A45" s="1" t="s">
         <v>43</v>
       </c>
@@ -2719,7 +2716,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="46" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="46" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A46" s="1" t="s">
         <v>44</v>
       </c>
@@ -2736,7 +2733,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="47" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="47" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A47" s="1" t="s">
         <v>45</v>
       </c>
@@ -2756,7 +2753,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="48" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="48" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A48" s="1" t="s">
         <v>46</v>
       </c>
@@ -2776,7 +2773,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="49" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="49" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A49" s="1" t="s">
         <v>47</v>
       </c>
@@ -2793,7 +2790,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="50" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="50" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A50" s="1" t="s">
         <v>48</v>
       </c>
@@ -2810,7 +2807,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="51" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="51" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A51" s="1" t="s">
         <v>49</v>
       </c>
@@ -2827,7 +2824,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="52" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="52" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A52" s="1" t="s">
         <v>50</v>
       </c>
@@ -2844,7 +2841,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="53" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="53" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A53" s="1" t="s">
         <v>51</v>
       </c>
@@ -2861,7 +2858,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="54" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="54" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A54" s="1" t="s">
         <v>52</v>
       </c>
@@ -2878,7 +2875,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="55" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="55" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A55" s="1" t="s">
         <v>53</v>
       </c>
@@ -2895,7 +2892,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="56" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="56" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A56" s="1" t="s">
         <v>54</v>
       </c>
@@ -2912,7 +2909,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="57" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="57" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A57" s="1" t="s">
         <v>55</v>
       </c>
@@ -2929,7 +2926,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="58" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="58" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A58" s="1" t="s">
         <v>56</v>
       </c>
@@ -2946,7 +2943,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="59" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="59" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A59" s="1" t="s">
         <v>57</v>
       </c>
@@ -2966,7 +2963,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="60" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="60" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A60" s="1" t="s">
         <v>58</v>
       </c>
@@ -2983,7 +2980,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="61" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="61" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A61" s="1" t="s">
         <v>59</v>
       </c>
@@ -3000,7 +2997,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="62" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="62" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A62" s="1" t="s">
         <v>60</v>
       </c>
@@ -3020,7 +3017,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="63" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="63" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A63" s="1" t="s">
         <v>61</v>
       </c>
@@ -3037,7 +3034,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="64" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="64" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A64" s="1" t="s">
         <v>62</v>
       </c>
@@ -3054,7 +3051,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="65" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A65" s="1" t="s">
         <v>63</v>
       </c>
@@ -3071,7 +3068,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="66" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A66" s="1" t="s">
         <v>64</v>
       </c>
@@ -3088,7 +3085,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="67" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A67" s="1" t="s">
         <v>65</v>
       </c>
@@ -3108,7 +3105,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="68" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A68" s="1" t="s">
         <v>66</v>
       </c>
@@ -3125,7 +3122,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="69" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A69" s="1" t="s">
         <v>67</v>
       </c>
@@ -3142,7 +3139,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="70" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A70" s="1" t="s">
         <v>68</v>
       </c>
@@ -3162,7 +3159,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="71" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A71" s="1" t="s">
         <v>69</v>
       </c>
@@ -3182,7 +3179,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="72" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A72" s="1" t="s">
         <v>70</v>
       </c>
@@ -3202,7 +3199,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="73" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A73" s="1" t="s">
         <v>71</v>
       </c>
@@ -3219,7 +3216,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="74" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A74" s="1" t="s">
         <v>72</v>
       </c>
@@ -3236,7 +3233,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="75" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A75" s="1" t="s">
         <v>73</v>
       </c>
@@ -3256,7 +3253,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="76" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A76" s="1" t="s">
         <v>74</v>
       </c>
@@ -3276,7 +3273,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A77" s="1" t="s">
         <v>75</v>
       </c>
@@ -3293,7 +3290,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="78" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A78" s="1" t="s">
         <v>76</v>
       </c>
@@ -3310,7 +3307,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="79" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A79" s="1" t="s">
         <v>77</v>
       </c>
@@ -3327,7 +3324,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="80" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A80" s="1" t="s">
         <v>78</v>
       </c>
@@ -3344,7 +3341,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="81" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="81" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A81" s="1" t="s">
         <v>79</v>
       </c>
@@ -3361,7 +3358,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="82" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="82" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A82" s="1" t="s">
         <v>80</v>
       </c>
@@ -3378,7 +3375,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="83" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="83" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A83" s="1" t="s">
         <v>81</v>
       </c>
@@ -3395,7 +3392,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="84" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="84" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A84" s="1" t="s">
         <v>82</v>
       </c>
@@ -3412,7 +3409,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="85" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="85" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A85" s="1" t="s">
         <v>83</v>
       </c>
@@ -3429,7 +3426,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="86" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="86" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A86" s="1" t="s">
         <v>84</v>
       </c>
@@ -3446,7 +3443,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="87" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="87" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A87" s="1" t="s">
         <v>85</v>
       </c>
@@ -3463,7 +3460,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="88" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="88" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A88" s="1" t="s">
         <v>86</v>
       </c>
@@ -3480,7 +3477,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="89" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="89" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A89" s="1" t="s">
         <v>87</v>
       </c>
@@ -3497,7 +3494,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="90" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="90" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A90" s="1" t="s">
         <v>88</v>
       </c>
@@ -3514,7 +3511,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="91" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="91" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A91" s="1" t="s">
         <v>89</v>
       </c>
@@ -3531,7 +3528,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="92" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="92" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A92" s="1" t="s">
         <v>90</v>
       </c>
@@ -3548,7 +3545,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="93" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="93" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A93" s="1" t="s">
         <v>91</v>
       </c>
@@ -3565,7 +3562,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="94" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="94" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A94" s="1" t="s">
         <v>92</v>
       </c>
@@ -3582,7 +3579,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="95" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="95" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A95" s="1" t="s">
         <v>93</v>
       </c>
@@ -3599,7 +3596,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="96" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="96" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A96" s="1" t="s">
         <v>94</v>
       </c>
@@ -3616,7 +3613,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="97" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A97" s="1" t="s">
         <v>95</v>
       </c>
@@ -3633,7 +3630,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="98" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A98" s="1" t="s">
         <v>96</v>
       </c>
@@ -3650,7 +3647,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="99" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A99" s="1" t="s">
         <v>97</v>
       </c>
@@ -3670,7 +3667,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="100" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A100" s="1" t="s">
         <v>98</v>
       </c>
@@ -3690,7 +3687,7 @@
         <v>349</v>
       </c>
     </row>
-    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="101" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A101" s="1" t="s">
         <v>99</v>
       </c>
@@ -3707,7 +3704,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="102" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A102" s="1" t="s">
         <v>100</v>
       </c>
@@ -3724,7 +3721,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="103" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A103" s="1" t="s">
         <v>101</v>
       </c>
@@ -3741,7 +3738,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="104" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A104" s="1" t="s">
         <v>102</v>
       </c>
@@ -3758,7 +3755,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="105" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A105" s="1" t="s">
         <v>103</v>
       </c>
@@ -3775,7 +3772,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="106" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A106" s="1" t="s">
         <v>104</v>
       </c>
@@ -3792,7 +3789,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="107" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A107" s="1" t="s">
         <v>105</v>
       </c>
@@ -3809,7 +3806,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="108" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A108" s="1" t="s">
         <v>106</v>
       </c>
@@ -3826,7 +3823,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="109" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A109" s="1" t="s">
         <v>107</v>
       </c>
@@ -3843,7 +3840,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="110" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A110" s="1" t="s">
         <v>108</v>
       </c>
@@ -3860,7 +3857,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="111" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A111" s="1" t="s">
         <v>109</v>
       </c>
@@ -3877,7 +3874,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="112" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A112" s="1" t="s">
         <v>110</v>
       </c>
@@ -3894,7 +3891,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="113" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A113" s="1" t="s">
         <v>111</v>
       </c>
@@ -3911,7 +3908,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="114" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A114" s="1" t="s">
         <v>112</v>
       </c>
@@ -3928,7 +3925,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="115" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A115" s="1" t="s">
         <v>113</v>
       </c>
@@ -3945,7 +3942,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="116" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A116" s="1" t="s">
         <v>114</v>
       </c>
@@ -3962,7 +3959,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="117" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A117" s="1" t="s">
         <v>115</v>
       </c>
@@ -3979,7 +3976,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="118" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A118" s="1" t="s">
         <v>116</v>
       </c>
@@ -3996,7 +3993,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="119" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A119" s="1" t="s">
         <v>117</v>
       </c>
@@ -4013,7 +4010,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="120" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A120" s="1" t="s">
         <v>118</v>
       </c>
@@ -4030,7 +4027,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="121" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A121" s="1" t="s">
         <v>119</v>
       </c>
@@ -4047,7 +4044,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="122" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A122" s="1" t="s">
         <v>120</v>
       </c>
@@ -4064,7 +4061,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="123" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A123" s="1" t="s">
         <v>121</v>
       </c>
@@ -4081,7 +4078,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="124" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A124" s="1" t="s">
         <v>122</v>
       </c>
@@ -4098,7 +4095,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="125" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A125" s="1" t="s">
         <v>123</v>
       </c>
@@ -4115,7 +4112,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A126" s="1" t="s">
         <v>124</v>
       </c>
@@ -4132,7 +4129,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="127" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A127" s="1" t="s">
         <v>125</v>
       </c>
@@ -4149,7 +4146,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="128" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A128" s="1" t="s">
         <v>126</v>
       </c>
@@ -4166,7 +4163,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="129" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A129" s="1" t="s">
         <v>127</v>
       </c>
@@ -4183,7 +4180,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="130" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A130" s="1" t="s">
         <v>128</v>
       </c>
@@ -4200,7 +4197,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="131" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A131" s="1" t="s">
         <v>129</v>
       </c>
@@ -4217,7 +4214,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="132" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A132" s="1" t="s">
         <v>130</v>
       </c>
@@ -4234,7 +4231,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="133" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A133" s="1" t="s">
         <v>131</v>
       </c>
@@ -4251,7 +4248,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="134" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A134" s="1" t="s">
         <v>132</v>
       </c>
@@ -4268,7 +4265,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="135" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="135" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A135" s="1" t="s">
         <v>133</v>
       </c>
@@ -4285,7 +4282,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="136" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="136" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A136" s="1" t="s">
         <v>134</v>
       </c>
@@ -4302,7 +4299,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="137" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="137" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A137" s="1" t="s">
         <v>135</v>
       </c>
@@ -4319,7 +4316,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="138" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="138" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A138" s="1" t="s">
         <v>136</v>
       </c>
@@ -4336,7 +4333,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="139" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="139" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A139" s="1" t="s">
         <v>137</v>
       </c>
@@ -4353,7 +4350,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="140" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="140" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A140" s="1" t="s">
         <v>138</v>
       </c>
@@ -4370,7 +4367,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="141" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="141" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A141" s="1" t="s">
         <v>139</v>
       </c>
@@ -4387,7 +4384,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="142" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="142" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A142" s="1" t="s">
         <v>140</v>
       </c>
@@ -4404,7 +4401,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="143" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="143" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A143" s="1" t="s">
         <v>141</v>
       </c>
@@ -4421,7 +4418,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="144" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="144" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A144" s="1" t="s">
         <v>142</v>
       </c>
@@ -4438,7 +4435,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="145" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="145" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A145" s="1" t="s">
         <v>143</v>
       </c>
@@ -4455,7 +4452,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="146" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="146" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A146" s="1" t="s">
         <v>144</v>
       </c>
@@ -4472,7 +4469,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="147" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="147" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A147" s="1" t="s">
         <v>145</v>
       </c>
@@ -4489,7 +4486,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="148" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="148" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A148" s="1" t="s">
         <v>146</v>
       </c>
@@ -4506,7 +4503,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="149" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="149" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A149" s="1" t="s">
         <v>147</v>
       </c>
@@ -4523,7 +4520,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="150" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="150" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A150" s="1" t="s">
         <v>148</v>
       </c>
@@ -4540,7 +4537,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="151" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="151" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A151" s="1" t="s">
         <v>149</v>
       </c>
@@ -4557,7 +4554,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="152" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="152" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A152" s="1" t="s">
         <v>150</v>
       </c>
@@ -4574,7 +4571,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="153" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="153" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A153" s="1" t="s">
         <v>151</v>
       </c>
@@ -4591,7 +4588,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="154" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="154" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A154" s="1" t="s">
         <v>152</v>
       </c>
@@ -4608,7 +4605,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="155" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="155" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A155" s="1" t="s">
         <v>153</v>
       </c>
@@ -4625,7 +4622,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="156" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="156" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A156" s="1" t="s">
         <v>154</v>
       </c>
@@ -4642,7 +4639,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="157" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="157" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A157" s="1" t="s">
         <v>155</v>
       </c>
@@ -4659,7 +4656,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="158" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="158" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A158" s="1" t="s">
         <v>156</v>
       </c>
@@ -4676,7 +4673,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="159" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="159" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A159" s="1" t="s">
         <v>157</v>
       </c>
@@ -4693,7 +4690,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="160" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="160" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A160" s="1" t="s">
         <v>158</v>
       </c>
@@ -4710,7 +4707,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="161" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A161" s="1" t="s">
         <v>159</v>
       </c>
@@ -4727,7 +4724,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="162" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A162" s="1" t="s">
         <v>160</v>
       </c>
@@ -4744,7 +4741,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="163" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A163" s="1" t="s">
         <v>161</v>
       </c>
@@ -4761,7 +4758,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="164" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A164" s="1" t="s">
         <v>162</v>
       </c>
@@ -4778,7 +4775,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="165" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A165" s="1" t="s">
         <v>163</v>
       </c>
@@ -4795,7 +4792,7 @@
         <v>347</v>
       </c>
     </row>
-    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
+    <row r="166" spans="1:6" x14ac:dyDescent="0.2">
       <c r="A166" s="1" t="s">
         <v>164</v>
       </c>
@@ -4821,21 +4818,21 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{531F7735-F42E-498C-BEC1-50736A9A963F}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="3" width="8.77734375" style="1"/>
-    <col min="4" max="4" width="49.77734375" style="1" bestFit="1" customWidth="1"/>
-    <col min="5" max="16384" width="8.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="3" width="8.83203125" style="1"/>
+    <col min="4" max="4" width="49.83203125" style="1" bestFit="1" customWidth="1"/>
+    <col min="5" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>358</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>359</v>
       </c>
@@ -4843,7 +4840,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>360</v>
       </c>
@@ -4851,7 +4848,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>361</v>
       </c>
@@ -4859,7 +4856,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>404</v>
       </c>
@@ -4867,7 +4864,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="7" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
         <v>403</v>
       </c>
@@ -4875,12 +4872,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="2" t="s">
         <v>362</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>363</v>
       </c>
@@ -4888,7 +4885,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>364</v>
       </c>
@@ -4896,7 +4893,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>365</v>
       </c>
@@ -4904,17 +4901,17 @@
         <v>402</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="1" t="s">
         <v>366</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="2" t="s">
         <v>367</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>368</v>
       </c>
@@ -4922,7 +4919,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>369</v>
       </c>
@@ -4938,20 +4935,20 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D46D2D27-EE5A-3443-81FE-8FFE2856088E}">
   <dimension ref="B2:C17"/>
-  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>370</v>
       </c>
       <c r="C2" s="2"/>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>371</v>
       </c>
@@ -4959,7 +4956,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>372</v>
       </c>
@@ -4967,7 +4964,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>373</v>
       </c>
@@ -4975,7 +4972,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>374</v>
       </c>
@@ -4983,12 +4980,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>375</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>376</v>
       </c>
@@ -4996,7 +4993,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>377</v>
       </c>
@@ -5004,7 +5001,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>378</v>
       </c>
@@ -5012,7 +5009,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="12" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="12" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B12" s="1" t="s">
         <v>379</v>
       </c>
@@ -5020,12 +5017,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" s="2" t="s">
         <v>380</v>
       </c>
     </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>381</v>
       </c>
@@ -5033,7 +5030,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>382</v>
       </c>
@@ -5041,7 +5038,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="17" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="17" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B17" s="1" t="s">
         <v>383</v>
       </c>
@@ -5057,19 +5054,19 @@
 <file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{45B0DAC4-B4F8-774F-9BF6-792E26EC6276}">
   <dimension ref="B2:C16"/>
-  <sheetFormatPr defaultColWidth="10.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="10.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="10.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="10.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>384</v>
       </c>
     </row>
-    <row r="3" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>387</v>
       </c>
@@ -5077,7 +5074,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="4" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>385</v>
       </c>
@@ -5085,7 +5082,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="5" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>388</v>
       </c>
@@ -5093,7 +5090,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="6" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>386</v>
       </c>
@@ -5101,12 +5098,12 @@
         <v>402</v>
       </c>
     </row>
-    <row r="8" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="8" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B8" s="2" t="s">
         <v>389</v>
       </c>
     </row>
-    <row r="9" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="9" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B9" s="1" t="s">
         <v>390</v>
       </c>
@@ -5114,7 +5111,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="10" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="10" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B10" s="1" t="s">
         <v>391</v>
       </c>
@@ -5122,7 +5119,7 @@
         <v>402</v>
       </c>
     </row>
-    <row r="11" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="11" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B11" s="1" t="s">
         <v>392</v>
       </c>
@@ -5130,22 +5127,25 @@
         <v>402</v>
       </c>
     </row>
-    <row r="13" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="13" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B13" s="2" t="s">
         <v>393</v>
       </c>
     </row>
-    <row r="14" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="14" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B14" s="1" t="s">
         <v>394</v>
       </c>
-    </row>
-    <row r="15" spans="2:3" x14ac:dyDescent="0.3">
+      <c r="C14" s="1" t="s">
+        <v>402</v>
+      </c>
+    </row>
+    <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>395</v>
       </c>
     </row>
-    <row r="16" spans="2:3" x14ac:dyDescent="0.3">
+    <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
         <v>396</v>
       </c>
@@ -5158,34 +5158,34 @@
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BB7FF8-2BA0-4E37-9F78-C30173234A80}">
   <dimension ref="B2:B6"/>
-  <sheetFormatPr defaultColWidth="8.77734375" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="1" width="5.77734375" style="1" customWidth="1"/>
-    <col min="2" max="2" width="100.77734375" style="1" customWidth="1"/>
-    <col min="3" max="16384" width="8.77734375" style="1"/>
+    <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
+    <col min="2" max="2" width="100.83203125" style="1" customWidth="1"/>
+    <col min="3" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
         <v>397</v>
       </c>
     </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B3" s="1" t="s">
         <v>398</v>
       </c>
     </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B4" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B5" s="1" t="s">
         <v>400</v>
       </c>
     </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.3">
+    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
         <v>401</v>
       </c>

</xml_diff>

<commit_message>
analisi terminata, scrivere relazione
</commit_message>
<xml_diff>
--- a/metadati.xlsx
+++ b/metadati.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/eca/Documents/data_analisi/progetto_g2/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D3422682-1BF7-724D-ADF6-8E56FBCCE6C6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5EC95564-ED1E-7443-841A-AF3879BB5F3A}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="660" windowWidth="23260" windowHeight="12460" tabRatio="860" activeTab="3" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
+    <workbookView xWindow="0" yWindow="660" windowWidth="29400" windowHeight="16960" tabRatio="860" activeTab="4" xr2:uid="{0B4D574E-D8BE-442B-A57A-A2F576E1D345}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata" sheetId="1" r:id="rId1"/>
@@ -48,7 +48,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="925" uniqueCount="405">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="929" uniqueCount="405">
   <si>
     <t>gameid</t>
   </si>
@@ -1466,9 +1466,6 @@
     <t>Quali player hanno la maggiore varianza di performance (partite molto buone vs molto negative)?</t>
   </si>
   <si>
-    <t>Esistono player “clutch” con migliori performance nelle partite lunghe (&gt;35 min)?</t>
-  </si>
-  <si>
     <t>Domande avanzate</t>
   </si>
   <si>
@@ -1514,6 +1511,9 @@
   </si>
   <si>
     <t>la percentuale di vittorie Blue side vs red side varia tra i vari split?</t>
+  </si>
+  <si>
+    <t>Esistono player “clutch” con migliori percformance nelle partite lunghe (&gt;35 min)?</t>
   </si>
 </sst>
 </file>
@@ -4837,7 +4837,7 @@
         <v>359</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
@@ -4845,7 +4845,7 @@
         <v>360</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
@@ -4853,23 +4853,23 @@
         <v>361</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B6" s="1" t="s">
-        <v>404</v>
+        <v>403</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="7" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B7" s="1" t="s">
-        <v>403</v>
+        <v>402</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="9" spans="2:3" x14ac:dyDescent="0.2">
@@ -4882,7 +4882,7 @@
         <v>363</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.2">
@@ -4890,7 +4890,7 @@
         <v>364</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
@@ -4898,7 +4898,7 @@
         <v>365</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.2">
@@ -4916,7 +4916,7 @@
         <v>368</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.2">
@@ -4924,7 +4924,7 @@
         <v>369</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -4953,7 +4953,7 @@
         <v>371</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
@@ -4961,7 +4961,7 @@
         <v>372</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
@@ -4969,7 +4969,7 @@
         <v>373</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
@@ -4977,7 +4977,7 @@
         <v>374</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
@@ -4990,7 +4990,7 @@
         <v>376</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.2">
@@ -4998,7 +4998,7 @@
         <v>377</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.2">
@@ -5006,7 +5006,7 @@
         <v>378</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="12" spans="2:3" x14ac:dyDescent="0.2">
@@ -5014,7 +5014,7 @@
         <v>379</v>
       </c>
       <c r="C12" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="14" spans="2:3" x14ac:dyDescent="0.2">
@@ -5027,7 +5027,7 @@
         <v>381</v>
       </c>
       <c r="C15" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.2">
@@ -5035,7 +5035,7 @@
         <v>382</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="17" spans="2:3" x14ac:dyDescent="0.2">
@@ -5043,7 +5043,7 @@
         <v>383</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -5071,7 +5071,7 @@
         <v>387</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="4" spans="2:3" x14ac:dyDescent="0.2">
@@ -5079,7 +5079,7 @@
         <v>385</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="5" spans="2:3" x14ac:dyDescent="0.2">
@@ -5087,7 +5087,7 @@
         <v>388</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="6" spans="2:3" x14ac:dyDescent="0.2">
@@ -5095,7 +5095,7 @@
         <v>386</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="8" spans="2:3" x14ac:dyDescent="0.2">
@@ -5108,7 +5108,7 @@
         <v>390</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="10" spans="2:3" x14ac:dyDescent="0.2">
@@ -5116,7 +5116,7 @@
         <v>391</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="11" spans="2:3" x14ac:dyDescent="0.2">
@@ -5124,7 +5124,7 @@
         <v>392</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="13" spans="2:3" x14ac:dyDescent="0.2">
@@ -5137,17 +5137,23 @@
         <v>394</v>
       </c>
       <c r="C14" s="1" t="s">
-        <v>402</v>
+        <v>401</v>
       </c>
     </row>
     <row r="15" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B15" s="1" t="s">
         <v>395</v>
       </c>
+      <c r="C15" s="1" t="s">
+        <v>401</v>
+      </c>
     </row>
     <row r="16" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B16" s="1" t="s">
-        <v>396</v>
+        <v>404</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>401</v>
       </c>
     </row>
   </sheetData>
@@ -5157,7 +5163,7 @@
 
 <file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{73BB7FF8-2BA0-4E37-9F78-C30173234A80}">
-  <dimension ref="B2:B6"/>
+  <dimension ref="B2:C6"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="5.83203125" style="1" customWidth="1"/>
@@ -5165,29 +5171,35 @@
     <col min="3" max="16384" width="8.83203125" style="1"/>
   </cols>
   <sheetData>
-    <row r="2" spans="2:2" x14ac:dyDescent="0.2">
+    <row r="2" spans="2:3" x14ac:dyDescent="0.2">
       <c r="B2" s="2" t="s">
+        <v>396</v>
+      </c>
+    </row>
+    <row r="3" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B3" s="1" t="s">
         <v>397</v>
       </c>
-    </row>
-    <row r="3" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B3" s="1" t="s">
+      <c r="C3" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="4" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B4" s="1" t="s">
         <v>398</v>
       </c>
-    </row>
-    <row r="4" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B4" s="1" t="s">
+      <c r="C4" s="1" t="s">
+        <v>401</v>
+      </c>
+    </row>
+    <row r="5" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B5" s="1" t="s">
         <v>399</v>
       </c>
     </row>
-    <row r="5" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B5" s="1" t="s">
+    <row r="6" spans="2:3" x14ac:dyDescent="0.2">
+      <c r="B6" s="1" t="s">
         <v>400</v>
-      </c>
-    </row>
-    <row r="6" spans="2:2" x14ac:dyDescent="0.2">
-      <c r="B6" s="1" t="s">
-        <v>401</v>
       </c>
     </row>
   </sheetData>

</xml_diff>